<commit_message>
Mise Ã  jour simulateur ROV
</commit_message>
<xml_diff>
--- a/simulateur_rov/Simu flottabilité.xlsx
+++ b/simulateur_rov/Simu flottabilité.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/338bbbaa6367577a/Documents/Projet ROV/simulateur_rov/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D5D2605-E06E-44E4-985D-6F3BB3C84330}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C00E8102-2D9F-428F-89CE-7DF8F4292E09}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DB299C8F-BC93-4B03-82ED-EDC1EFAE3C08}"/>
   </bookViews>
@@ -205,12 +205,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -226,7 +232,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -237,6 +243,10 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -1773,7 +1783,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D864BA-B9B5-4F28-AD0C-D9CA645A41BB}">
   <sheetPr codeName="Feuil1"/>
-  <dimension ref="C1:AB24"/>
+  <dimension ref="C1:AB31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.28515625" customWidth="1"/>
@@ -2116,7 +2126,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="5">
-        <v>3.5000000000000003E-2</v>
+        <v>0.03</v>
       </c>
       <c r="E8" t="s">
         <v>18</v>
@@ -2227,19 +2237,19 @@
       </c>
       <c r="D10" s="5">
         <f>D8*D1*D2</f>
-        <v>353.65050000000002</v>
+        <v>303.12900000000002</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="11" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="9">
         <f>D10+D9</f>
-        <v>59.350500000000011</v>
+        <v>8.8290000000000077</v>
       </c>
       <c r="E11" t="s">
         <v>11</v>
@@ -2557,7 +2567,7 @@
       </c>
       <c r="D17" s="6">
         <f>SQRT(ABS(2*D11/(D2*D13*D15)))</f>
-        <v>0.67625160070927648</v>
+        <v>0.26082659599079294</v>
       </c>
       <c r="E17" t="s">
         <v>16</v>
@@ -2619,6 +2629,26 @@
       </c>
       <c r="E24" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D28">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="29" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D29">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="30" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D30">
+        <v>13.77</v>
+      </c>
+    </row>
+    <row r="31" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D31">
+        <v>8.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mise Ã  jour simulateur et corrections cÃ¢ble
</commit_message>
<xml_diff>
--- a/simulateur_rov/Simu flottabilité.xlsx
+++ b/simulateur_rov/Simu flottabilité.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/338bbbaa6367577a/Documents/Projet ROV/simulateur_rov/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C00E8102-2D9F-428F-89CE-7DF8F4292E09}"/>
+  <xr:revisionPtr revIDLastSave="223" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C6DD242-0C2E-470B-B8D6-1FAB9A997769}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DB299C8F-BC93-4B03-82ED-EDC1EFAE3C08}"/>
+    <workbookView minimized="1" xWindow="4860" yWindow="-15120" windowWidth="21600" windowHeight="11295" xr2:uid="{DB299C8F-BC93-4B03-82ED-EDC1EFAE3C08}"/>
   </bookViews>
   <sheets>
     <sheet name="Traînée ROV" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
   <si>
     <t>Cy</t>
   </si>
@@ -172,7 +172,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.0000_-;\-* #,##0.0000_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -240,13 +240,13 @@
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -2631,24 +2631,38 @@
         <v>11</v>
       </c>
     </row>
+    <row r="27" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27">
+        <v>0.13</v>
+      </c>
+    </row>
     <row r="28" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D28">
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="29" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D29">
-        <v>0.4</v>
+      <c r="C28" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="7">
+        <f>0.5*$D$12*$D$14*D27*D27*$D$2</f>
+        <v>1.2533040000000006</v>
       </c>
     </row>
     <row r="30" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>24</v>
+      </c>
       <c r="D30">
-        <v>13.77</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="31" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D31">
-        <v>8.83</v>
+      <c r="C31" t="s">
+        <v>32</v>
+      </c>
+      <c r="D31" s="7">
+        <f>0.5*$D$13*$D$15*D30*D30*$D$2</f>
+        <v>124.64071199999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout assertions invariants cable et doc tests
</commit_message>
<xml_diff>
--- a/simulateur_rov/Simu flottabilité.xlsx
+++ b/simulateur_rov/Simu flottabilité.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/338bbbaa6367577a/Documents/Projet ROV/simulateur_rov/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="223" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C6DD242-0C2E-470B-B8D6-1FAB9A997769}"/>
+  <xr:revisionPtr revIDLastSave="422" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE30BA5C-BBA6-4303-970E-373A0E788D76}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4860" yWindow="-15120" windowWidth="21600" windowHeight="11295" xr2:uid="{DB299C8F-BC93-4B03-82ED-EDC1EFAE3C08}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DB299C8F-BC93-4B03-82ED-EDC1EFAE3C08}"/>
   </bookViews>
   <sheets>
-    <sheet name="Traînée ROV" sheetId="1" r:id="rId1"/>
-    <sheet name="Feuil1" sheetId="5" r:id="rId2"/>
+    <sheet name="Data envt" sheetId="5" r:id="rId1"/>
+    <sheet name="Traînée ROV" sheetId="1" r:id="rId2"/>
+    <sheet name="Traînée courant" sheetId="6" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="53">
   <si>
     <t>Cy</t>
   </si>
@@ -161,6 +162,63 @@
   </si>
   <si>
     <t>V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROV </t>
+  </si>
+  <si>
+    <t>CABLE</t>
+  </si>
+  <si>
+    <t>Cf</t>
+  </si>
+  <si>
+    <t>Longueur cable</t>
+  </si>
+  <si>
+    <t>Surface_x</t>
+  </si>
+  <si>
+    <t>Surface_y</t>
+  </si>
+  <si>
+    <t>Fond _y</t>
+  </si>
+  <si>
+    <t>Fond_x</t>
+  </si>
+  <si>
+    <t>teta</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>u</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>V courant</t>
+  </si>
+  <si>
+    <t>V cable</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Trainée long</t>
+  </si>
+  <si>
+    <t>Trainée perp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trainée cable </t>
   </si>
 </sst>
 </file>
@@ -174,7 +232,7 @@
     <numFmt numFmtId="166" formatCode="_-* #,##0.0000_-;\-* #,##0.0000_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -204,8 +262,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -215,6 +281,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -232,7 +310,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -247,6 +325,14 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -254,6 +340,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFFCC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1781,9 +1872,287 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF37EC3C-F57F-4626-8718-178BD2240E14}">
+  <sheetPr codeName="Feuil4"/>
+  <dimension ref="A3:C30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3">
+        <v>9.81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1030</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="5">
+        <v>0.7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="5">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="5">
+        <v>0.03</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="5">
+        <f>-1*B10*B3</f>
+        <v>-294.3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="5">
+        <f>B11*B3*B4</f>
+        <v>303.12900000000002</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="9">
+        <f>B13+B12</f>
+        <v>8.8290000000000077</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="11">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="11">
+        <v>0.9</v>
+      </c>
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="5">
+        <f>B7*B9</f>
+        <v>0.16000000000000003</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="5">
+        <f>B7*B8</f>
+        <v>0.27999999999999997</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="6">
+        <f>SQRT(ABS(2*B14/(B4*B16*B18)))</f>
+        <v>0.26082659599079294</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="6"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="6"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="4">
+        <v>1E-3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="3">
+        <v>950</v>
+      </c>
+      <c r="C24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" s="4">
+        <f>B3*B24*PI()*POWER(B23,2)/4</f>
+        <v>7.3195181837825193E-3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="4" cm="1">
+        <f t="array" ref="B26">B3*(B24-B4)*PI()*POWER(B23:B23,2)/4</f>
+        <v>-6.1638047863431743E-4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="4">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" s="4">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="4">
+        <f>100*B26</f>
+        <v>-6.1638047863431744E-2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D864BA-B9B5-4F28-AD0C-D9CA645A41BB}">
   <sheetPr codeName="Feuil1"/>
-  <dimension ref="C1:AB31"/>
+  <dimension ref="C4:AB13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.28515625" customWidth="1"/>
@@ -1791,41 +2160,12 @@
     <col min="8" max="28" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3">
-        <v>9.81</v>
-      </c>
-      <c r="E1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="3">
-        <v>1030</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
-    </row>
     <row r="4" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="5">
-        <v>0.4</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4">
+        <v>0.13</v>
       </c>
       <c r="G4" t="s">
         <v>23</v>
@@ -1915,123 +2255,107 @@
       </c>
     </row>
     <row r="5" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="5">
-        <v>0.7</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="7">
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*D4*D4*'Data envt'!$B$4</f>
+        <v>1.2533040000000006</v>
       </c>
       <c r="G5" t="s">
         <v>31</v>
       </c>
       <c r="H5" s="7">
-        <f>0.5*$D$12*$D$14*H4*H4*$D$2</f>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*H4*H4*'Data envt'!$B$4</f>
         <v>0</v>
       </c>
       <c r="I5" s="7">
-        <f>0.5*$D$12*$D$14*I4*I4*$D$2</f>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*I4*I4*'Data envt'!$B$4</f>
         <v>0.74160000000000026</v>
       </c>
       <c r="J5" s="7">
-        <f t="shared" ref="J5:AB5" si="3">0.5*$D$12*$D$14*J4*J4*$D$2</f>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*J4*J4*'Data envt'!$B$4</f>
         <v>2.966400000000001</v>
       </c>
       <c r="K5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*K4*K4*'Data envt'!$B$4</f>
         <v>6.6744000000000048</v>
       </c>
       <c r="L5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*L4*L4*'Data envt'!$B$4</f>
         <v>11.865600000000004</v>
       </c>
       <c r="M5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*M4*M4*'Data envt'!$B$4</f>
         <v>18.540000000000006</v>
       </c>
       <c r="N5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*N4*N4*'Data envt'!$B$4</f>
         <v>26.697600000000005</v>
       </c>
       <c r="O5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*O4*O4*'Data envt'!$B$4</f>
         <v>36.338400000000007</v>
       </c>
       <c r="P5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*P4*P4*'Data envt'!$B$4</f>
         <v>47.462400000000002</v>
       </c>
       <c r="Q5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*Q4*Q4*'Data envt'!$B$4</f>
         <v>60.069600000000001</v>
       </c>
       <c r="R5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*R4*R4*'Data envt'!$B$4</f>
         <v>74.16</v>
       </c>
       <c r="S5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*S4*S4*'Data envt'!$B$4</f>
         <v>89.733600000000024</v>
       </c>
       <c r="T5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*T4*T4*'Data envt'!$B$4</f>
         <v>106.79040000000002</v>
       </c>
       <c r="U5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*U4*U4*'Data envt'!$B$4</f>
         <v>125.33040000000004</v>
       </c>
       <c r="V5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*V4*V4*'Data envt'!$B$4</f>
         <v>145.35360000000009</v>
       </c>
       <c r="W5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*W4*W4*'Data envt'!$B$4</f>
         <v>166.86000000000013</v>
       </c>
       <c r="X5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*X4*X4*'Data envt'!$B$4</f>
         <v>189.84960000000012</v>
       </c>
       <c r="Y5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*Y4*Y4*'Data envt'!$B$4</f>
         <v>214.32240000000016</v>
       </c>
       <c r="Z5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*Z4*Z4*'Data envt'!$B$4</f>
         <v>240.2784000000002</v>
       </c>
       <c r="AA5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*AA4*AA4*'Data envt'!$B$4</f>
         <v>267.71760000000029</v>
       </c>
       <c r="AB5" s="7">
-        <f t="shared" si="3"/>
+        <f>0.5*'Data envt'!$B$15*'Data envt'!$B$17*AB4*AB4*'Data envt'!$B$4</f>
         <v>296.64000000000021</v>
       </c>
     </row>
-    <row r="6" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="5">
-        <v>0.4</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-    </row>
     <row r="7" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="5">
-        <v>30</v>
-      </c>
-      <c r="E7" t="s">
-        <v>17</v>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7">
+        <v>0.9</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" t="s">
@@ -2045,214 +2369,188 @@
         <v>0.1</v>
       </c>
       <c r="J7">
-        <f t="shared" ref="J7:AB7" si="4">I7+0.1</f>
+        <f t="shared" ref="J7:AB7" si="3">I7+0.1</f>
         <v>0.2</v>
       </c>
       <c r="K7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="L7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0.4</v>
       </c>
       <c r="M7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="N7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="O7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0.7</v>
       </c>
       <c r="P7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0.79999999999999993</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0.89999999999999991</v>
       </c>
       <c r="R7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0.99999999999999989</v>
       </c>
       <c r="S7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.0999999999999999</v>
       </c>
       <c r="T7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.2</v>
       </c>
       <c r="U7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.3</v>
       </c>
       <c r="V7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.4000000000000001</v>
       </c>
       <c r="W7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.5000000000000002</v>
       </c>
       <c r="X7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.6000000000000003</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.7000000000000004</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.8000000000000005</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.9000000000000006</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.0000000000000004</v>
       </c>
     </row>
     <row r="8" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C8" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="5">
-        <v>0.03</v>
-      </c>
-      <c r="E8" t="s">
-        <v>18</v>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="7">
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*D7*D7*'Data envt'!$B$4</f>
+        <v>105.12179999999999</v>
       </c>
       <c r="G8" t="s">
         <v>32</v>
       </c>
       <c r="H8" s="7">
-        <f>0.5*$D$13*$D$15*H7*H7*$D$2</f>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*H7*H7*'Data envt'!$B$4</f>
         <v>0</v>
       </c>
       <c r="I8" s="7">
-        <f>0.5*$D$13*$D$15*I7*I7*$D$2</f>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*I7*I7*'Data envt'!$B$4</f>
         <v>1.2978000000000001</v>
       </c>
       <c r="J8" s="7">
-        <f t="shared" ref="J8:AB8" si="5">0.5*$D$13*$D$15*J7*J7*$D$2</f>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*J7*J7*'Data envt'!$B$4</f>
         <v>5.1912000000000003</v>
       </c>
       <c r="K8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*K7*K7*'Data envt'!$B$4</f>
         <v>11.680200000000005</v>
       </c>
       <c r="L8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*L7*L7*'Data envt'!$B$4</f>
         <v>20.764800000000001</v>
       </c>
       <c r="M8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*M7*M7*'Data envt'!$B$4</f>
         <v>32.445</v>
       </c>
       <c r="N8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*N7*N7*'Data envt'!$B$4</f>
         <v>46.720799999999997</v>
       </c>
       <c r="O8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*O7*O7*'Data envt'!$B$4</f>
         <v>63.592199999999998</v>
       </c>
       <c r="P8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*P7*P7*'Data envt'!$B$4</f>
         <v>83.05919999999999</v>
       </c>
       <c r="Q8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*Q7*Q7*'Data envt'!$B$4</f>
         <v>105.12179999999998</v>
       </c>
       <c r="R8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*R7*R7*'Data envt'!$B$4</f>
         <v>129.77999999999994</v>
       </c>
       <c r="S8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*S7*S7*'Data envt'!$B$4</f>
         <v>157.03379999999996</v>
       </c>
       <c r="T8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*T7*T7*'Data envt'!$B$4</f>
         <v>186.88319999999999</v>
       </c>
       <c r="U8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*U7*U7*'Data envt'!$B$4</f>
         <v>219.32820000000001</v>
       </c>
       <c r="V8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*V7*V7*'Data envt'!$B$4</f>
         <v>254.36880000000008</v>
       </c>
       <c r="W8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*W7*W7*'Data envt'!$B$4</f>
         <v>292.00500000000011</v>
       </c>
       <c r="X8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*X7*X7*'Data envt'!$B$4</f>
         <v>332.23680000000013</v>
       </c>
       <c r="Y8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*Y7*Y7*'Data envt'!$B$4</f>
         <v>375.0642000000002</v>
       </c>
       <c r="Z8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*Z7*Z7*'Data envt'!$B$4</f>
         <v>420.4872000000002</v>
       </c>
       <c r="AA8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*AA7*AA7*'Data envt'!$B$4</f>
         <v>468.50580000000031</v>
       </c>
       <c r="AB8" s="7">
-        <f t="shared" si="5"/>
+        <f>0.5*'Data envt'!$B$16*'Data envt'!$B$18*AB7*AB7*'Data envt'!$B$4</f>
         <v>519.12000000000023</v>
       </c>
     </row>
-    <row r="9" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="5">
-        <f>-1*D7*D1</f>
-        <v>-294.3</v>
-      </c>
-      <c r="E9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C10" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" s="5">
-        <f>D8*D1*D2</f>
-        <v>303.12900000000002</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
-      </c>
-    </row>
     <row r="11" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C11" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="9">
-        <f>D10+D9</f>
-        <v>8.8290000000000077</v>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="6">
+        <f>'Data envt'!B20</f>
+        <v>0.26082659599079294</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G11" t="s">
         <v>33</v>
@@ -2262,93 +2560,87 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <f t="shared" ref="I11:AB11" si="6">I4</f>
+        <f t="shared" ref="I11:AB11" si="4">I4</f>
         <v>0.1</v>
       </c>
       <c r="J11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.2</v>
       </c>
       <c r="K11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="L11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.4</v>
       </c>
       <c r="M11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.5</v>
       </c>
       <c r="N11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.6</v>
       </c>
       <c r="O11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.7</v>
       </c>
       <c r="P11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.79999999999999993</v>
       </c>
       <c r="Q11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.89999999999999991</v>
       </c>
       <c r="R11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.99999999999999989</v>
       </c>
       <c r="S11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.0999999999999999</v>
       </c>
       <c r="T11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.2</v>
       </c>
       <c r="U11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.3</v>
       </c>
       <c r="V11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.4000000000000001</v>
       </c>
       <c r="W11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.5000000000000002</v>
       </c>
       <c r="X11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.6000000000000003</v>
       </c>
       <c r="Y11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.7000000000000004</v>
       </c>
       <c r="Z11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.8000000000000005</v>
       </c>
       <c r="AA11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>1.9000000000000006</v>
       </c>
       <c r="AB11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>2.0000000000000004</v>
       </c>
     </row>
     <row r="12" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="5">
-        <v>0.9</v>
-      </c>
       <c r="G12" t="s">
         <v>31</v>
       </c>
@@ -2357,94 +2649,87 @@
         <v>0</v>
       </c>
       <c r="I12" s="7">
-        <f t="shared" ref="I12:AB12" si="7">I5</f>
+        <f t="shared" ref="I12:AB12" si="5">I5</f>
         <v>0.74160000000000026</v>
       </c>
       <c r="J12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>2.966400000000001</v>
       </c>
       <c r="K12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>6.6744000000000048</v>
       </c>
       <c r="L12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>11.865600000000004</v>
       </c>
       <c r="M12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>18.540000000000006</v>
       </c>
       <c r="N12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>26.697600000000005</v>
       </c>
       <c r="O12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>36.338400000000007</v>
       </c>
       <c r="P12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>47.462400000000002</v>
       </c>
       <c r="Q12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>60.069600000000001</v>
       </c>
       <c r="R12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>74.16</v>
       </c>
       <c r="S12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>89.733600000000024</v>
       </c>
       <c r="T12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>106.79040000000002</v>
       </c>
       <c r="U12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>125.33040000000004</v>
       </c>
       <c r="V12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>145.35360000000009</v>
       </c>
       <c r="W12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>166.86000000000013</v>
       </c>
       <c r="X12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>189.84960000000012</v>
       </c>
       <c r="Y12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>214.32240000000016</v>
       </c>
       <c r="Z12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>240.2784000000002</v>
       </c>
       <c r="AA12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>267.71760000000029</v>
       </c>
       <c r="AB12" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>296.64000000000021</v>
       </c>
     </row>
     <row r="13" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5">
-        <v>0.9</v>
-      </c>
-      <c r="E13" s="1"/>
       <c r="G13" t="s">
         <v>32</v>
       </c>
@@ -2453,216 +2738,84 @@
         <v>0</v>
       </c>
       <c r="I13" s="7">
-        <f t="shared" ref="I13:AB13" si="8">I8</f>
+        <f t="shared" ref="I13:AB13" si="6">I8</f>
         <v>1.2978000000000001</v>
       </c>
       <c r="J13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>5.1912000000000003</v>
       </c>
       <c r="K13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>11.680200000000005</v>
       </c>
       <c r="L13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>20.764800000000001</v>
       </c>
       <c r="M13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>32.445</v>
       </c>
       <c r="N13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46.720799999999997</v>
       </c>
       <c r="O13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>63.592199999999998</v>
       </c>
       <c r="P13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>83.05919999999999</v>
       </c>
       <c r="Q13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>105.12179999999998</v>
       </c>
       <c r="R13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>129.77999999999994</v>
       </c>
       <c r="S13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>157.03379999999996</v>
       </c>
       <c r="T13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>186.88319999999999</v>
       </c>
       <c r="U13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>219.32820000000001</v>
       </c>
       <c r="V13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>254.36880000000008</v>
       </c>
       <c r="W13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>292.00500000000011</v>
       </c>
       <c r="X13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>332.23680000000013</v>
       </c>
       <c r="Y13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>375.0642000000002</v>
       </c>
       <c r="Z13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>420.4872000000002</v>
       </c>
       <c r="AA13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>468.50580000000031</v>
       </c>
       <c r="AB13" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>519.12000000000023</v>
-      </c>
-    </row>
-    <row r="14" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="5">
-        <f>D4*D6</f>
-        <v>0.16000000000000003</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="5">
-        <f>D4*D5</f>
-        <v>0.27999999999999997</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="3:28" x14ac:dyDescent="0.25">
-      <c r="C16" s="2"/>
-      <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C17" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" s="6">
-        <f>SQRT(ABS(2*D11/(D2*D13*D15)))</f>
-        <v>0.26082659599079294</v>
-      </c>
-      <c r="E17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="4">
-        <v>1E-3</v>
-      </c>
-      <c r="E19" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C20" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="3">
-        <v>1500</v>
-      </c>
-      <c r="E20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C21" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="4">
-        <f>D20*PI()*POWER(D19,2)/4</f>
-        <v>1.1780972450961724E-3</v>
-      </c>
-      <c r="E21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C22" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="4" cm="1">
-        <f t="array" ref="D22">(D20-D2)*PI()*POWER(D19:D19,2)/4</f>
-        <v>3.6913713679680068E-4</v>
-      </c>
-      <c r="E22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C24" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D24" s="4">
-        <f>100*D22</f>
-        <v>3.691371367968007E-2</v>
-      </c>
-      <c r="E24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C27" t="s">
-        <v>23</v>
-      </c>
-      <c r="D27">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="28" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C28" t="s">
-        <v>31</v>
-      </c>
-      <c r="D28" s="7">
-        <f>0.5*$D$12*$D$14*D27*D27*$D$2</f>
-        <v>1.2533040000000006</v>
-      </c>
-    </row>
-    <row r="30" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C30" t="s">
-        <v>24</v>
-      </c>
-      <c r="D30">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="31" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C31" t="s">
-        <v>32</v>
-      </c>
-      <c r="D31" s="7">
-        <f>0.5*$D$13*$D$15*D30*D30*$D$2</f>
-        <v>124.64071199999999</v>
       </c>
     </row>
   </sheetData>
@@ -2671,16 +2824,362 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF37EC3C-F57F-4626-8718-178BD2240E14}">
-  <sheetPr codeName="Feuil4"/>
-  <dimension ref="D25"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15A5C9A5-74C6-40F1-8B51-97BB0A88B95F}">
+  <sheetPr codeName="Feuil2"/>
+  <dimension ref="A2:J30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="25" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D25">
-        <f>SQRT(104)</f>
-        <v>10.198039027185569</v>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H2" t="str">
+        <f>'Data envt'!A4</f>
+        <v xml:space="preserve">Rho </v>
+      </c>
+      <c r="I2">
+        <f>'Data envt'!B4</f>
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H4" t="str">
+        <f>'Data envt'!A22</f>
+        <v>CABLE</v>
+      </c>
+      <c r="I4">
+        <f>'Data envt'!B22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="str">
+        <f>'Data envt'!A23</f>
+        <v>Diamètre câble</v>
+      </c>
+      <c r="I5">
+        <f>'Data envt'!B23</f>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="str">
+        <f>'Data envt'!A24</f>
+        <v>Masse volumique</v>
+      </c>
+      <c r="I6">
+        <f>'Data envt'!B24</f>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="str">
+        <f>'Data envt'!A25</f>
+        <v>Poids linéique</v>
+      </c>
+      <c r="I7">
+        <f>'Data envt'!B25</f>
+        <v>7.3195181837825193E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8">
+        <v>400</v>
+      </c>
+      <c r="H8" t="str">
+        <f>'Data envt'!A26</f>
+        <v>Poids apparent linéique</v>
+      </c>
+      <c r="I8">
+        <f>'Data envt'!B26</f>
+        <v>-6.1638047863431743E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9">
+        <f>SQRT(POWER(B7-B5,2)+POWER(B8-B6,2))</f>
+        <v>400</v>
+      </c>
+      <c r="H9" t="str">
+        <f>'Data envt'!A27</f>
+        <v>Cx</v>
+      </c>
+      <c r="I9">
+        <f>'Data envt'!B27</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10">
+        <f>ASIN(B7/B9)</f>
+        <v>0</v>
+      </c>
+      <c r="H10" t="str">
+        <f>'Data envt'!A28</f>
+        <v>Cf</v>
+      </c>
+      <c r="I10">
+        <f>'Data envt'!B28</f>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H11">
+        <f>'Data envt'!A29</f>
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <f>'Data envt'!B29</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12">
+        <f>SIN(B10)</f>
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12">
+        <f>-COS(B10)</f>
+        <v>-1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" t="str">
+        <f>'Data envt'!A30</f>
+        <v>Poids apparent 100 m</v>
+      </c>
+      <c r="I12">
+        <f>'Data envt'!B30</f>
+        <v>-6.1638047863431744E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13">
+        <f>COS(B10)</f>
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13">
+        <f>SIN(B10)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H14" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14">
+        <v>400</v>
+      </c>
+      <c r="J14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15">
+        <f>SIN(B10)</f>
+        <v>0</v>
+      </c>
+      <c r="C15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15">
+        <f>-COS(B10)</f>
+        <v>-1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16">
+        <f>COS(B10)</f>
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16">
+        <f>SIN(B10)</f>
+        <v>0</v>
+      </c>
+      <c r="E16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="13">
+        <v>0</v>
+      </c>
+      <c r="C18" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="13">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <f>B15*B18</f>
+        <v>0</v>
+      </c>
+      <c r="C19" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19">
+        <f>D15*B18</f>
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="13">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="13">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23">
+        <f>0.5*I9*I2*I5*D19*ABS(D19)*I14</f>
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24">
+        <f>0.5*I10*I2*PI()*I5*(B19+B21)*ABS(B19+B21)*I14</f>
+        <v>25.886723465579902</v>
+      </c>
+      <c r="C24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27">
+        <f>D23*B13</f>
+        <v>0</v>
+      </c>
+      <c r="C27" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27">
+        <f>D23*D13</f>
+        <v>0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28">
+        <f>B24*B12</f>
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28">
+        <f>B24*D12</f>
+        <v>-25.886723465579902</v>
+      </c>
+      <c r="E28" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <f>B27+B28</f>
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <f>D27+D28</f>
+        <v>-25.886723465579902</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simulateur ROV: tests UI, traînée bornée, câble et missions
- Onglet Tests: pytest sans capture stdout/stderr (traces visibles dans le terminal)
- ROV: saturation des vitesses pour la traînée (évite overflow v*|v|); clip vx/vy pour forces dans system_model
- Tests: test_rov_model extrêmes, catalogues et visuels câble; cable_snapshot_dialog, cable_hover
- Nettoyage traces et fichiers mission locaux (M100/M101/M102/M_unit_*)
- Divers: conftest, pytest.ini, simulation_tab/thread, plotter, utils, xlsx flottabilité

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/simulateur_rov/Simu flottabilité.xlsx
+++ b/simulateur_rov/Simu flottabilité.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/338bbbaa6367577a/Documents/Projet ROV/simulateur_rov/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="422" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE30BA5C-BBA6-4303-970E-373A0E788D76}"/>
+  <xr:revisionPtr revIDLastSave="433" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EDCD08C-43AD-4AED-ABDC-7FC30D134632}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DB299C8F-BC93-4B03-82ED-EDC1EFAE3C08}"/>
   </bookViews>
   <sheets>
     <sheet name="Data envt" sheetId="5" r:id="rId1"/>
     <sheet name="Traînée ROV" sheetId="1" r:id="rId2"/>
-    <sheet name="Traînée courant" sheetId="6" r:id="rId3"/>
+    <sheet name="Traînée câble" sheetId="6" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1552,10 +1552,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>

</xml_diff>

<commit_message>
Simulateur ROV: intégration projetée DAE, init missions, catalogue Tests UI
- Intégrateur half-explicit (projected_integrator), projection d'état, spec DAE

- Conditions initiales strict/legacy, missions M_test_init_*, tests non-régression

- Catalogue onglet Tests (src/tests/test_catalog.py), docs régénérée et script regenerate_documentation

- Ajustements M103, environnement, câble, UI simulation et tracés

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/simulateur_rov/Simu flottabilité.xlsx
+++ b/simulateur_rov/Simu flottabilité.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/338bbbaa6367577a/Documents/Projet ROV/simulateur_rov/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="433" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EDCD08C-43AD-4AED-ABDC-7FC30D134632}"/>
+  <xr:revisionPtr revIDLastSave="599" documentId="13_ncr:1_{B2A7D9EE-2791-4AA6-9F58-AE3493008ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A25D67A-FF6C-4146-ABCF-196779139894}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DB299C8F-BC93-4B03-82ED-EDC1EFAE3C08}"/>
+    <workbookView xWindow="660" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{DB299C8F-BC93-4B03-82ED-EDC1EFAE3C08}"/>
   </bookViews>
   <sheets>
     <sheet name="Data envt" sheetId="5" r:id="rId1"/>
     <sheet name="Traînée ROV" sheetId="1" r:id="rId2"/>
     <sheet name="Traînée câble" sheetId="6" r:id="rId3"/>
+    <sheet name="Initialisation" sheetId="7" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="67">
   <si>
     <t>Cy</t>
   </si>
@@ -219,6 +220,48 @@
   </si>
   <si>
     <t xml:space="preserve">Trainée cable </t>
+  </si>
+  <si>
+    <t>xrov</t>
+  </si>
+  <si>
+    <t>yrov</t>
+  </si>
+  <si>
+    <t>L_straight</t>
+  </si>
+  <si>
+    <t>xH</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>xH + L</t>
+  </si>
+  <si>
+    <t>L init</t>
+  </si>
+  <si>
+    <t>| xH + L - L_init |</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>a min</t>
+  </si>
+  <si>
+    <t>xH min</t>
+  </si>
+  <si>
+    <t>L arc</t>
+  </si>
+  <si>
+    <t>a ach((yrov+a)/a)</t>
   </si>
 </sst>
 </file>
@@ -310,7 +353,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -333,6 +376,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -1552,6 +1596,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -1946,7 +1994,7 @@
         <v>12</v>
       </c>
       <c r="B10" s="5">
-        <v>30</v>
+        <v>30.9</v>
       </c>
       <c r="C10" t="s">
         <v>17</v>
@@ -1969,7 +2017,7 @@
       </c>
       <c r="B12" s="5">
         <f>-1*B10*B3</f>
-        <v>-294.3</v>
+        <v>-303.12900000000002</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
@@ -1993,7 +2041,7 @@
       </c>
       <c r="B14" s="9">
         <f>B13+B12</f>
-        <v>8.8290000000000077</v>
+        <v>0</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
@@ -2050,7 +2098,7 @@
       </c>
       <c r="B20" s="6">
         <f>SQRT(ABS(2*B14/(B4*B16*B18)))</f>
-        <v>0.26082659599079294</v>
+        <v>0</v>
       </c>
       <c r="C20" t="s">
         <v>16</v>
@@ -2081,7 +2129,7 @@
         <v>15</v>
       </c>
       <c r="B24" s="3">
-        <v>950</v>
+        <v>1030</v>
       </c>
       <c r="C24" t="s">
         <v>19</v>
@@ -2093,7 +2141,7 @@
       </c>
       <c r="B25" s="4">
         <f>B3*B24*PI()*POWER(B23,2)/4</f>
-        <v>7.3195181837825193E-3</v>
+        <v>7.9358986624168369E-3</v>
       </c>
       <c r="C25" t="s">
         <v>7</v>
@@ -2105,7 +2153,7 @@
       </c>
       <c r="B26" s="4" cm="1">
         <f t="array" ref="B26">B3*(B24-B4)*PI()*POWER(B23:B23,2)/4</f>
-        <v>-6.1638047863431743E-4</v>
+        <v>0</v>
       </c>
       <c r="C26" t="s">
         <v>7</v>
@@ -2133,7 +2181,7 @@
       </c>
       <c r="B30" s="4">
         <f>100*B26</f>
-        <v>-6.1638047863431744E-2</v>
+        <v>0</v>
       </c>
       <c r="C30" t="s">
         <v>11</v>
@@ -2543,7 +2591,7 @@
       </c>
       <c r="D11" s="6">
         <f>'Data envt'!B20</f>
-        <v>0.26082659599079294</v>
+        <v>0</v>
       </c>
       <c r="E11" t="s">
         <v>16</v>
@@ -2879,7 +2927,7 @@
       </c>
       <c r="I6">
         <f>'Data envt'!B24</f>
-        <v>950</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -2895,7 +2943,7 @@
       </c>
       <c r="I7">
         <f>'Data envt'!B25</f>
-        <v>7.3195181837825193E-3</v>
+        <v>7.9358986624168369E-3</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -2911,7 +2959,7 @@
       </c>
       <c r="I8">
         <f>'Data envt'!B26</f>
-        <v>-6.1638047863431743E-4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -2982,7 +3030,7 @@
       </c>
       <c r="I12">
         <f>'Data envt'!B30</f>
-        <v>-6.1638047863431744E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -3058,7 +3106,7 @@
         <v>47</v>
       </c>
       <c r="B18" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" t="s">
         <v>43</v>
@@ -3080,7 +3128,7 @@
       </c>
       <c r="D19">
         <f>D15*B18</f>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E19" t="s">
         <v>46</v>
@@ -3091,7 +3139,7 @@
         <v>48</v>
       </c>
       <c r="B21" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" t="s">
         <v>45</v>
@@ -3109,7 +3157,7 @@
       </c>
       <c r="D23">
         <f>0.5*I9*I2*I5*D19*ABS(D19)*I14</f>
-        <v>0</v>
+        <v>-185.4</v>
       </c>
       <c r="E23" t="s">
         <v>46</v>
@@ -3121,7 +3169,7 @@
       </c>
       <c r="B24">
         <f>0.5*I10*I2*PI()*I5*(B19+B21)*ABS(B19+B21)*I14</f>
-        <v>25.886723465579902</v>
+        <v>0</v>
       </c>
       <c r="C24" t="s">
         <v>45</v>
@@ -3133,7 +3181,7 @@
       </c>
       <c r="B27">
         <f>D23*B13</f>
-        <v>0</v>
+        <v>-185.4</v>
       </c>
       <c r="C27" t="s">
         <v>43</v>
@@ -3159,7 +3207,7 @@
       </c>
       <c r="D28">
         <f>B24*D12</f>
-        <v>-25.886723465579902</v>
+        <v>0</v>
       </c>
       <c r="E28" t="s">
         <v>44</v>
@@ -3171,11 +3219,2529 @@
       </c>
       <c r="B30">
         <f>B27+B28</f>
-        <v>0</v>
+        <v>-185.4</v>
       </c>
       <c r="D30">
         <f>D27+D28</f>
-        <v>-25.886723465579902</v>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B278E61F-21F6-4C96-A7AC-8B91979F7E41}">
+  <sheetPr codeName="Feuil3"/>
+  <dimension ref="B2:DA13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="18.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <f>F2+1</f>
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <f t="shared" ref="H2:BH2" si="0">G2+1</f>
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="L2">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="M2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="N2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="O2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="P2">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="Q2">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="R2">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="S2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="T2">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="U2">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="V2">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="W2">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="X2">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="Y2">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="Z2">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="AA2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="AB2">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="AC2">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="AD2">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="AE2">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="AF2">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="AG2">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="AH2">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="AI2">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="AJ2">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="AK2">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="AL2">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="AM2">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="AN2">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="AO2">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="AP2">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+      <c r="AQ2">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="AR2">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="AS2">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="AT2">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="AU2">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="AV2">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="AW2">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="AX2">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="AY2">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="AZ2">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="BA2">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="BB2">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="BC2">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="BD2">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="BE2">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="BF2">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="BG2">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="BH2">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+      <c r="BI2">
+        <f t="shared" ref="BI2:BZ2" si="1">BH2+1</f>
+        <v>56</v>
+      </c>
+      <c r="BJ2">
+        <f t="shared" si="1"/>
+        <v>57</v>
+      </c>
+      <c r="BK2">
+        <f t="shared" si="1"/>
+        <v>58</v>
+      </c>
+      <c r="BL2">
+        <f t="shared" si="1"/>
+        <v>59</v>
+      </c>
+      <c r="BM2">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="BN2">
+        <f t="shared" si="1"/>
+        <v>61</v>
+      </c>
+      <c r="BO2">
+        <f t="shared" si="1"/>
+        <v>62</v>
+      </c>
+      <c r="BP2">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="BQ2">
+        <f t="shared" si="1"/>
+        <v>64</v>
+      </c>
+      <c r="BR2">
+        <f t="shared" si="1"/>
+        <v>65</v>
+      </c>
+      <c r="BS2">
+        <f t="shared" si="1"/>
+        <v>66</v>
+      </c>
+      <c r="BT2">
+        <f t="shared" si="1"/>
+        <v>67</v>
+      </c>
+      <c r="BU2">
+        <f t="shared" si="1"/>
+        <v>68</v>
+      </c>
+      <c r="BV2">
+        <f t="shared" si="1"/>
+        <v>69</v>
+      </c>
+      <c r="BW2">
+        <f t="shared" si="1"/>
+        <v>70</v>
+      </c>
+      <c r="BX2">
+        <f t="shared" si="1"/>
+        <v>71</v>
+      </c>
+      <c r="BY2">
+        <f t="shared" si="1"/>
+        <v>72</v>
+      </c>
+      <c r="BZ2">
+        <f t="shared" si="1"/>
+        <v>73</v>
+      </c>
+      <c r="CA2">
+        <f t="shared" ref="CA2:DA2" si="2">BZ2+1</f>
+        <v>74</v>
+      </c>
+      <c r="CB2">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+      <c r="CC2">
+        <f t="shared" si="2"/>
+        <v>76</v>
+      </c>
+      <c r="CD2">
+        <f t="shared" si="2"/>
+        <v>77</v>
+      </c>
+      <c r="CE2">
+        <f t="shared" si="2"/>
+        <v>78</v>
+      </c>
+      <c r="CF2">
+        <f t="shared" si="2"/>
+        <v>79</v>
+      </c>
+      <c r="CG2">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="CH2">
+        <f t="shared" si="2"/>
+        <v>81</v>
+      </c>
+      <c r="CI2">
+        <f t="shared" si="2"/>
+        <v>82</v>
+      </c>
+      <c r="CJ2">
+        <f t="shared" si="2"/>
+        <v>83</v>
+      </c>
+      <c r="CK2">
+        <f t="shared" si="2"/>
+        <v>84</v>
+      </c>
+      <c r="CL2">
+        <f t="shared" si="2"/>
+        <v>85</v>
+      </c>
+      <c r="CM2">
+        <f t="shared" si="2"/>
+        <v>86</v>
+      </c>
+      <c r="CN2">
+        <f t="shared" si="2"/>
+        <v>87</v>
+      </c>
+      <c r="CO2">
+        <f t="shared" si="2"/>
+        <v>88</v>
+      </c>
+      <c r="CP2">
+        <f t="shared" si="2"/>
+        <v>89</v>
+      </c>
+      <c r="CQ2">
+        <f t="shared" si="2"/>
+        <v>90</v>
+      </c>
+      <c r="CR2">
+        <f t="shared" si="2"/>
+        <v>91</v>
+      </c>
+      <c r="CS2">
+        <f t="shared" si="2"/>
+        <v>92</v>
+      </c>
+      <c r="CT2">
+        <f t="shared" si="2"/>
+        <v>93</v>
+      </c>
+      <c r="CU2">
+        <f t="shared" si="2"/>
+        <v>94</v>
+      </c>
+      <c r="CV2">
+        <f t="shared" si="2"/>
+        <v>95</v>
+      </c>
+      <c r="CW2">
+        <f t="shared" si="2"/>
+        <v>96</v>
+      </c>
+      <c r="CX2">
+        <f t="shared" si="2"/>
+        <v>97</v>
+      </c>
+      <c r="CY2">
+        <f t="shared" si="2"/>
+        <v>98</v>
+      </c>
+      <c r="CZ2">
+        <f t="shared" si="2"/>
+        <v>99</v>
+      </c>
+      <c r="DA2">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4">
+        <v>400</v>
+      </c>
+      <c r="E4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4">
+        <v>0.01</v>
+      </c>
+      <c r="G4">
+        <f>F4+0.2</f>
+        <v>0.21000000000000002</v>
+      </c>
+      <c r="H4">
+        <f t="shared" ref="H4:U4" si="3">G4+0.2</f>
+        <v>0.41000000000000003</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="3"/>
+        <v>0.6100000000000001</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="3"/>
+        <v>0.81</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="3"/>
+        <v>1.01</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="3"/>
+        <v>1.21</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="3"/>
+        <v>1.41</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="3"/>
+        <v>1.6099999999999999</v>
+      </c>
+      <c r="O4">
+        <f t="shared" si="3"/>
+        <v>1.8099999999999998</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="3"/>
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" si="3"/>
+        <v>2.21</v>
+      </c>
+      <c r="R4">
+        <f t="shared" si="3"/>
+        <v>2.41</v>
+      </c>
+      <c r="S4">
+        <f t="shared" si="3"/>
+        <v>2.6100000000000003</v>
+      </c>
+      <c r="T4">
+        <f t="shared" si="3"/>
+        <v>2.8100000000000005</v>
+      </c>
+      <c r="U4">
+        <f t="shared" si="3"/>
+        <v>3.0100000000000007</v>
+      </c>
+      <c r="V4">
+        <f t="shared" ref="V4:AU4" si="4">U4+0.2</f>
+        <v>3.2100000000000009</v>
+      </c>
+      <c r="W4">
+        <f t="shared" si="4"/>
+        <v>3.410000000000001</v>
+      </c>
+      <c r="X4">
+        <f t="shared" si="4"/>
+        <v>3.6100000000000012</v>
+      </c>
+      <c r="Y4">
+        <f t="shared" si="4"/>
+        <v>3.8100000000000014</v>
+      </c>
+      <c r="Z4">
+        <f t="shared" si="4"/>
+        <v>4.0100000000000016</v>
+      </c>
+      <c r="AA4">
+        <f t="shared" si="4"/>
+        <v>4.2100000000000017</v>
+      </c>
+      <c r="AB4">
+        <f t="shared" si="4"/>
+        <v>4.4100000000000019</v>
+      </c>
+      <c r="AC4">
+        <f t="shared" si="4"/>
+        <v>4.6100000000000021</v>
+      </c>
+      <c r="AD4">
+        <f t="shared" si="4"/>
+        <v>4.8100000000000023</v>
+      </c>
+      <c r="AE4">
+        <f t="shared" si="4"/>
+        <v>5.0100000000000025</v>
+      </c>
+      <c r="AF4">
+        <f t="shared" si="4"/>
+        <v>5.2100000000000026</v>
+      </c>
+      <c r="AG4">
+        <f t="shared" si="4"/>
+        <v>5.4100000000000028</v>
+      </c>
+      <c r="AH4">
+        <f t="shared" si="4"/>
+        <v>5.610000000000003</v>
+      </c>
+      <c r="AI4">
+        <f t="shared" si="4"/>
+        <v>5.8100000000000032</v>
+      </c>
+      <c r="AJ4">
+        <f t="shared" si="4"/>
+        <v>6.0100000000000033</v>
+      </c>
+      <c r="AK4">
+        <f t="shared" si="4"/>
+        <v>6.2100000000000035</v>
+      </c>
+      <c r="AL4">
+        <f t="shared" si="4"/>
+        <v>6.4100000000000037</v>
+      </c>
+      <c r="AM4">
+        <f t="shared" si="4"/>
+        <v>6.6100000000000039</v>
+      </c>
+      <c r="AN4">
+        <f t="shared" si="4"/>
+        <v>6.8100000000000041</v>
+      </c>
+      <c r="AO4">
+        <f t="shared" si="4"/>
+        <v>7.0100000000000042</v>
+      </c>
+      <c r="AP4">
+        <f t="shared" si="4"/>
+        <v>7.2100000000000044</v>
+      </c>
+      <c r="AQ4">
+        <f t="shared" si="4"/>
+        <v>7.4100000000000046</v>
+      </c>
+      <c r="AR4">
+        <f t="shared" si="4"/>
+        <v>7.6100000000000048</v>
+      </c>
+      <c r="AS4">
+        <f t="shared" si="4"/>
+        <v>7.8100000000000049</v>
+      </c>
+      <c r="AT4">
+        <f t="shared" si="4"/>
+        <v>8.0100000000000051</v>
+      </c>
+      <c r="AU4">
+        <f t="shared" si="4"/>
+        <v>8.2100000000000044</v>
+      </c>
+      <c r="AV4">
+        <f t="shared" ref="AV4" si="5">AU4+0.2</f>
+        <v>8.4100000000000037</v>
+      </c>
+      <c r="AW4">
+        <f t="shared" ref="AW4" si="6">AV4+0.2</f>
+        <v>8.610000000000003</v>
+      </c>
+      <c r="AX4">
+        <f t="shared" ref="AX4" si="7">AW4+0.2</f>
+        <v>8.8100000000000023</v>
+      </c>
+      <c r="AY4">
+        <f t="shared" ref="AY4" si="8">AX4+0.2</f>
+        <v>9.0100000000000016</v>
+      </c>
+      <c r="AZ4">
+        <f t="shared" ref="AZ4" si="9">AY4+0.2</f>
+        <v>9.2100000000000009</v>
+      </c>
+      <c r="BA4">
+        <f t="shared" ref="BA4" si="10">AZ4+0.2</f>
+        <v>9.41</v>
+      </c>
+      <c r="BB4">
+        <f t="shared" ref="BB4" si="11">BA4+0.2</f>
+        <v>9.61</v>
+      </c>
+      <c r="BC4">
+        <f t="shared" ref="BC4" si="12">BB4+0.2</f>
+        <v>9.8099999999999987</v>
+      </c>
+      <c r="BD4">
+        <f t="shared" ref="BD4" si="13">BC4+0.2</f>
+        <v>10.009999999999998</v>
+      </c>
+      <c r="BE4">
+        <f t="shared" ref="BE4" si="14">BD4+0.2</f>
+        <v>10.209999999999997</v>
+      </c>
+      <c r="BF4">
+        <f t="shared" ref="BF4" si="15">BE4+0.2</f>
+        <v>10.409999999999997</v>
+      </c>
+      <c r="BG4">
+        <f t="shared" ref="BG4" si="16">BF4+0.2</f>
+        <v>10.609999999999996</v>
+      </c>
+      <c r="BH4">
+        <f t="shared" ref="BH4" si="17">BG4+0.2</f>
+        <v>10.809999999999995</v>
+      </c>
+      <c r="BI4">
+        <f t="shared" ref="BI4" si="18">BH4+0.2</f>
+        <v>11.009999999999994</v>
+      </c>
+      <c r="BJ4">
+        <f t="shared" ref="BJ4" si="19">BI4+0.2</f>
+        <v>11.209999999999994</v>
+      </c>
+      <c r="BK4">
+        <f t="shared" ref="BK4" si="20">BJ4+0.2</f>
+        <v>11.409999999999993</v>
+      </c>
+      <c r="BL4">
+        <f t="shared" ref="BL4" si="21">BK4+0.2</f>
+        <v>11.609999999999992</v>
+      </c>
+      <c r="BM4">
+        <f t="shared" ref="BM4" si="22">BL4+0.2</f>
+        <v>11.809999999999992</v>
+      </c>
+      <c r="BN4">
+        <f t="shared" ref="BN4" si="23">BM4+0.2</f>
+        <v>12.009999999999991</v>
+      </c>
+      <c r="BO4">
+        <f t="shared" ref="BO4" si="24">BN4+0.2</f>
+        <v>12.20999999999999</v>
+      </c>
+      <c r="BP4">
+        <f t="shared" ref="BP4" si="25">BO4+0.2</f>
+        <v>12.409999999999989</v>
+      </c>
+      <c r="BQ4">
+        <f t="shared" ref="BQ4" si="26">BP4+0.2</f>
+        <v>12.609999999999989</v>
+      </c>
+      <c r="BR4">
+        <f t="shared" ref="BR4" si="27">BQ4+0.2</f>
+        <v>12.809999999999988</v>
+      </c>
+      <c r="BS4">
+        <f t="shared" ref="BS4" si="28">BR4+0.2</f>
+        <v>13.009999999999987</v>
+      </c>
+      <c r="BT4">
+        <f t="shared" ref="BT4" si="29">BS4+0.2</f>
+        <v>13.209999999999987</v>
+      </c>
+      <c r="BU4">
+        <f t="shared" ref="BU4" si="30">BT4+0.2</f>
+        <v>13.409999999999986</v>
+      </c>
+      <c r="BV4">
+        <f t="shared" ref="BV4" si="31">BU4+0.2</f>
+        <v>13.609999999999985</v>
+      </c>
+      <c r="BW4">
+        <f t="shared" ref="BW4" si="32">BV4+0.2</f>
+        <v>13.809999999999985</v>
+      </c>
+      <c r="BX4">
+        <f t="shared" ref="BX4" si="33">BW4+0.2</f>
+        <v>14.009999999999984</v>
+      </c>
+      <c r="BY4">
+        <f t="shared" ref="BY4" si="34">BX4+0.2</f>
+        <v>14.209999999999983</v>
+      </c>
+      <c r="BZ4">
+        <f t="shared" ref="BZ4" si="35">BY4+0.2</f>
+        <v>14.409999999999982</v>
+      </c>
+      <c r="CA4">
+        <f t="shared" ref="CA4" si="36">BZ4+0.2</f>
+        <v>14.609999999999982</v>
+      </c>
+      <c r="CB4">
+        <f t="shared" ref="CB4" si="37">CA4+0.2</f>
+        <v>14.809999999999981</v>
+      </c>
+      <c r="CC4">
+        <f t="shared" ref="CC4" si="38">CB4+0.2</f>
+        <v>15.00999999999998</v>
+      </c>
+      <c r="CD4">
+        <f t="shared" ref="CD4" si="39">CC4+0.2</f>
+        <v>15.20999999999998</v>
+      </c>
+      <c r="CE4">
+        <f t="shared" ref="CE4" si="40">CD4+0.2</f>
+        <v>15.409999999999979</v>
+      </c>
+      <c r="CF4">
+        <f t="shared" ref="CF4" si="41">CE4+0.2</f>
+        <v>15.609999999999978</v>
+      </c>
+      <c r="CG4">
+        <f t="shared" ref="CG4" si="42">CF4+0.2</f>
+        <v>15.809999999999977</v>
+      </c>
+      <c r="CH4">
+        <f t="shared" ref="CH4" si="43">CG4+0.2</f>
+        <v>16.009999999999977</v>
+      </c>
+      <c r="CI4">
+        <f t="shared" ref="CI4" si="44">CH4+0.2</f>
+        <v>16.209999999999976</v>
+      </c>
+      <c r="CJ4">
+        <f t="shared" ref="CJ4" si="45">CI4+0.2</f>
+        <v>16.409999999999975</v>
+      </c>
+      <c r="CK4">
+        <f t="shared" ref="CK4" si="46">CJ4+0.2</f>
+        <v>16.609999999999975</v>
+      </c>
+      <c r="CL4">
+        <f t="shared" ref="CL4" si="47">CK4+0.2</f>
+        <v>16.809999999999974</v>
+      </c>
+      <c r="CM4">
+        <f t="shared" ref="CM4" si="48">CL4+0.2</f>
+        <v>17.009999999999973</v>
+      </c>
+      <c r="CN4">
+        <f t="shared" ref="CN4" si="49">CM4+0.2</f>
+        <v>17.209999999999972</v>
+      </c>
+      <c r="CO4">
+        <f t="shared" ref="CO4" si="50">CN4+0.2</f>
+        <v>17.409999999999972</v>
+      </c>
+      <c r="CP4">
+        <f t="shared" ref="CP4" si="51">CO4+0.2</f>
+        <v>17.609999999999971</v>
+      </c>
+      <c r="CQ4">
+        <f t="shared" ref="CQ4" si="52">CP4+0.2</f>
+        <v>17.80999999999997</v>
+      </c>
+      <c r="CR4">
+        <f t="shared" ref="CR4" si="53">CQ4+0.2</f>
+        <v>18.00999999999997</v>
+      </c>
+      <c r="CS4">
+        <f t="shared" ref="CS4" si="54">CR4+0.2</f>
+        <v>18.209999999999969</v>
+      </c>
+      <c r="CT4">
+        <f t="shared" ref="CT4" si="55">CS4+0.2</f>
+        <v>18.409999999999968</v>
+      </c>
+      <c r="CU4">
+        <f t="shared" ref="CU4" si="56">CT4+0.2</f>
+        <v>18.609999999999967</v>
+      </c>
+      <c r="CV4">
+        <f t="shared" ref="CV4" si="57">CU4+0.2</f>
+        <v>18.809999999999967</v>
+      </c>
+      <c r="CW4">
+        <f t="shared" ref="CW4" si="58">CV4+0.2</f>
+        <v>19.009999999999966</v>
+      </c>
+      <c r="CX4">
+        <f t="shared" ref="CX4" si="59">CW4+0.2</f>
+        <v>19.209999999999965</v>
+      </c>
+      <c r="CY4">
+        <f t="shared" ref="CY4" si="60">CX4+0.2</f>
+        <v>19.409999999999965</v>
+      </c>
+      <c r="CZ4">
+        <f t="shared" ref="CZ4" si="61">CY4+0.2</f>
+        <v>19.609999999999964</v>
+      </c>
+      <c r="DA4">
+        <f t="shared" ref="DA4" si="62">CZ4+0.2</f>
+        <v>19.809999999999963</v>
+      </c>
+    </row>
+    <row r="5" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5">
+        <v>420</v>
+      </c>
+      <c r="E5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5">
+        <f>$C$3-F4*ACOSH($C$4/F4 +1)</f>
+        <v>29.887101930868127</v>
+      </c>
+      <c r="G5">
+        <f t="shared" ref="G5:U5" si="63">$C$3-G4*ACOSH($C$4/G4 +1)</f>
+        <v>28.268385303439786</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="63"/>
+        <v>26.893334035449541</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="63"/>
+        <v>25.619936901989742</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="63"/>
+        <v>24.413142700762798</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="63"/>
+        <v>23.25604655524824</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="63"/>
+        <v>22.138618471039486</v>
+      </c>
+      <c r="M5">
+        <f t="shared" si="63"/>
+        <v>21.054201786048189</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="63"/>
+        <v>19.998051371866246</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="63"/>
+        <v>18.966611769608896</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="63"/>
+        <v>17.957118822927626</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" si="63"/>
+        <v>16.967361579027873</v>
+      </c>
+      <c r="R5">
+        <f t="shared" si="63"/>
+        <v>15.995531125379642</v>
+      </c>
+      <c r="S5">
+        <f t="shared" si="63"/>
+        <v>15.040119961154515</v>
+      </c>
+      <c r="T5">
+        <f t="shared" si="63"/>
+        <v>14.099852395478928</v>
+      </c>
+      <c r="U5">
+        <f t="shared" si="63"/>
+        <v>13.17363486076065</v>
+      </c>
+      <c r="V5">
+        <f t="shared" ref="V5" si="64">$C$3-V4*ACOSH($C$4/V4 +1)</f>
+        <v>12.260519488831218</v>
+      </c>
+      <c r="W5">
+        <f t="shared" ref="W5" si="65">$C$3-W4*ACOSH($C$4/W4 +1)</f>
+        <v>11.359676798759086</v>
+      </c>
+      <c r="X5">
+        <f t="shared" ref="X5" si="66">$C$3-X4*ACOSH($C$4/X4 +1)</f>
+        <v>10.470374813308158</v>
+      </c>
+      <c r="Y5">
+        <f t="shared" ref="Y5" si="67">$C$3-Y4*ACOSH($C$4/Y4 +1)</f>
+        <v>9.5919628168006952</v>
+      </c>
+      <c r="Z5">
+        <f t="shared" ref="Z5" si="68">$C$3-Z4*ACOSH($C$4/Z4 +1)</f>
+        <v>8.7238585322462576</v>
+      </c>
+      <c r="AA5">
+        <f t="shared" ref="AA5" si="69">$C$3-AA4*ACOSH($C$4/AA4 +1)</f>
+        <v>7.8655378625962591</v>
+      </c>
+      <c r="AB5">
+        <f t="shared" ref="AB5" si="70">$C$3-AB4*ACOSH($C$4/AB4 +1)</f>
+        <v>7.0165265854897285</v>
+      </c>
+      <c r="AC5">
+        <f t="shared" ref="AC5" si="71">$C$3-AC4*ACOSH($C$4/AC4 +1)</f>
+        <v>6.1763935574832338</v>
+      </c>
+      <c r="AD5">
+        <f t="shared" ref="AD5" si="72">$C$3-AD4*ACOSH($C$4/AD4 +1)</f>
+        <v>5.3447450996299573</v>
+      </c>
+      <c r="AE5">
+        <f t="shared" ref="AE5" si="73">$C$3-AE4*ACOSH($C$4/AE4 +1)</f>
+        <v>4.5212203183271633</v>
+      </c>
+      <c r="AF5">
+        <f t="shared" ref="AF5" si="74">$C$3-AF4*ACOSH($C$4/AF4 +1)</f>
+        <v>3.7054871744186357</v>
+      </c>
+      <c r="AG5">
+        <f t="shared" ref="AG5" si="75">$C$3-AG4*ACOSH($C$4/AG4 +1)</f>
+        <v>2.8972391566971503</v>
+      </c>
+      <c r="AH5">
+        <f t="shared" ref="AH5" si="76">$C$3-AH4*ACOSH($C$4/AH4 +1)</f>
+        <v>2.0961924479186713</v>
+      </c>
+      <c r="AI5">
+        <f t="shared" ref="AI5" si="77">$C$3-AI4*ACOSH($C$4/AI4 +1)</f>
+        <v>1.3020834954131537</v>
+      </c>
+      <c r="AJ5">
+        <f t="shared" ref="AJ5" si="78">$C$3-AJ4*ACOSH($C$4/AJ4 +1)</f>
+        <v>0.51466691656324315</v>
+      </c>
+      <c r="AK5">
+        <f t="shared" ref="AK5" si="79">$C$3-AK4*ACOSH($C$4/AK4 +1)</f>
+        <v>-0.26628631663531266</v>
+      </c>
+      <c r="AL5">
+        <f t="shared" ref="AL5" si="80">$C$3-AL4*ACOSH($C$4/AL4 +1)</f>
+        <v>-1.0409904589231012</v>
+      </c>
+      <c r="AM5">
+        <f t="shared" ref="AM5" si="81">$C$3-AM4*ACOSH($C$4/AM4 +1)</f>
+        <v>-1.8096463755947347</v>
+      </c>
+      <c r="AN5">
+        <f t="shared" ref="AN5" si="82">$C$3-AN4*ACOSH($C$4/AN4 +1)</f>
+        <v>-2.5724427586981236</v>
+      </c>
+      <c r="AO5">
+        <f t="shared" ref="AO5" si="83">$C$3-AO4*ACOSH($C$4/AO4 +1)</f>
+        <v>-3.3295572002520402</v>
+      </c>
+      <c r="AP5">
+        <f t="shared" ref="AP5" si="84">$C$3-AP4*ACOSH($C$4/AP4 +1)</f>
+        <v>-4.0811571428967284</v>
+      </c>
+      <c r="AQ5">
+        <f t="shared" ref="AQ5" si="85">$C$3-AQ4*ACOSH($C$4/AQ4 +1)</f>
+        <v>-4.8274007249911435</v>
+      </c>
+      <c r="AR5">
+        <f t="shared" ref="AR5" si="86">$C$3-AR4*ACOSH($C$4/AR4 +1)</f>
+        <v>-5.5684375344128512</v>
+      </c>
+      <c r="AS5">
+        <f t="shared" ref="AS5" si="87">$C$3-AS4*ACOSH($C$4/AS4 +1)</f>
+        <v>-6.3044092830663985</v>
+      </c>
+      <c r="AT5">
+        <f t="shared" ref="AT5" si="88">$C$3-AT4*ACOSH($C$4/AT4 +1)</f>
+        <v>-7.035450412259884</v>
+      </c>
+      <c r="AU5">
+        <f t="shared" ref="AU5:BH5" si="89">$C$3-AU4*ACOSH($C$4/AU4 +1)</f>
+        <v>-7.761688637586218</v>
+      </c>
+      <c r="AV5">
+        <f t="shared" si="89"/>
+        <v>-8.4832454406821824</v>
+      </c>
+      <c r="AW5">
+        <f t="shared" si="89"/>
+        <v>-9.2002365141856473</v>
+      </c>
+      <c r="AX5">
+        <f t="shared" si="89"/>
+        <v>-9.9127721653298551</v>
+      </c>
+      <c r="AY5">
+        <f t="shared" si="89"/>
+        <v>-10.620957682872323</v>
+      </c>
+      <c r="AZ5">
+        <f t="shared" si="89"/>
+        <v>-11.324893671429898</v>
+      </c>
+      <c r="BA5">
+        <f t="shared" si="89"/>
+        <v>-12.0246763567607</v>
+      </c>
+      <c r="BB5">
+        <f t="shared" si="89"/>
+        <v>-12.720397865081956</v>
+      </c>
+      <c r="BC5">
+        <f t="shared" si="89"/>
+        <v>-13.412146479126562</v>
+      </c>
+      <c r="BD5">
+        <f t="shared" si="89"/>
+        <v>-14.100006873310875</v>
+      </c>
+      <c r="BE5">
+        <f t="shared" si="89"/>
+        <v>-14.784060330101177</v>
+      </c>
+      <c r="BF5">
+        <f t="shared" si="89"/>
+        <v>-15.464384939421059</v>
+      </c>
+      <c r="BG5">
+        <f t="shared" si="89"/>
+        <v>-16.141055782729573</v>
+      </c>
+      <c r="BH5">
+        <f t="shared" si="89"/>
+        <v>-16.814145103215409</v>
+      </c>
+      <c r="BI5">
+        <f t="shared" ref="BI5:BZ5" si="90">$C$3-BI4*ACOSH($C$4/BI4 +1)</f>
+        <v>-17.483722463391864</v>
+      </c>
+      <c r="BJ5">
+        <f t="shared" si="90"/>
+        <v>-18.149854891237489</v>
+      </c>
+      <c r="BK5">
+        <f t="shared" si="90"/>
+        <v>-18.812607015904412</v>
+      </c>
+      <c r="BL5">
+        <f t="shared" si="90"/>
+        <v>-19.472041193909064</v>
+      </c>
+      <c r="BM5">
+        <f t="shared" si="90"/>
+        <v>-20.12821762662518</v>
+      </c>
+      <c r="BN5">
+        <f t="shared" si="90"/>
+        <v>-20.781194469815993</v>
+      </c>
+      <c r="BO5">
+        <f t="shared" si="90"/>
+        <v>-21.431027935868407</v>
+      </c>
+      <c r="BP5">
+        <f t="shared" si="90"/>
+        <v>-22.077772389327279</v>
+      </c>
+      <c r="BQ5">
+        <f t="shared" si="90"/>
+        <v>-22.721480436269566</v>
+      </c>
+      <c r="BR5">
+        <f t="shared" si="90"/>
+        <v>-23.362203008007263</v>
+      </c>
+      <c r="BS5">
+        <f t="shared" si="90"/>
+        <v>-23.999989439561702</v>
+      </c>
+      <c r="BT5">
+        <f t="shared" si="90"/>
+        <v>-24.634887543311429</v>
+      </c>
+      <c r="BU5">
+        <f t="shared" si="90"/>
+        <v>-25.266943678178905</v>
+      </c>
+      <c r="BV5">
+        <f t="shared" si="90"/>
+        <v>-25.896202814688891</v>
+      </c>
+      <c r="BW5">
+        <f t="shared" si="90"/>
+        <v>-26.52270859620203</v>
+      </c>
+      <c r="BX5">
+        <f t="shared" si="90"/>
+        <v>-27.146503396600323</v>
+      </c>
+      <c r="BY5">
+        <f t="shared" si="90"/>
+        <v>-27.767628374678161</v>
+      </c>
+      <c r="BZ5">
+        <f t="shared" si="90"/>
+        <v>-28.386123525470552</v>
+      </c>
+      <c r="CA5">
+        <f t="shared" ref="CA5:DA5" si="91">$C$3-CA4*ACOSH($C$4/CA4 +1)</f>
+        <v>-29.002027728731299</v>
+      </c>
+      <c r="CB5">
+        <f t="shared" si="91"/>
+        <v>-29.615378794756083</v>
+      </c>
+      <c r="CC5">
+        <f t="shared" si="91"/>
+        <v>-30.226213507729931</v>
+      </c>
+      <c r="CD5">
+        <f t="shared" si="91"/>
+        <v>-30.834567666763903</v>
+      </c>
+      <c r="CE5">
+        <f t="shared" si="91"/>
+        <v>-31.440476124772985</v>
+      </c>
+      <c r="CF5">
+        <f t="shared" si="91"/>
+        <v>-32.043972825335345</v>
+      </c>
+      <c r="CG5">
+        <f t="shared" si="91"/>
+        <v>-32.645090837662259</v>
+      </c>
+      <c r="CH5">
+        <f t="shared" si="91"/>
+        <v>-33.243862389798196</v>
+      </c>
+      <c r="CI5">
+        <f t="shared" si="91"/>
+        <v>-33.840318900161677</v>
+      </c>
+      <c r="CJ5">
+        <f t="shared" si="91"/>
+        <v>-34.434491007529303</v>
+      </c>
+      <c r="CK5">
+        <f t="shared" si="91"/>
+        <v>-35.026408599557712</v>
+      </c>
+      <c r="CL5">
+        <f t="shared" si="91"/>
+        <v>-35.616100839931704</v>
+      </c>
+      <c r="CM5">
+        <f t="shared" si="91"/>
+        <v>-36.20359619422004</v>
+      </c>
+      <c r="CN5">
+        <f t="shared" si="91"/>
+        <v>-36.788922454515145</v>
+      </c>
+      <c r="CO5">
+        <f t="shared" si="91"/>
+        <v>-37.372106762927146</v>
+      </c>
+      <c r="CP5">
+        <f t="shared" si="91"/>
+        <v>-37.9531756339982</v>
+      </c>
+      <c r="CQ5">
+        <f t="shared" si="91"/>
+        <v>-38.532154976098539</v>
+      </c>
+      <c r="CR5">
+        <f t="shared" si="91"/>
+        <v>-39.109070111861072</v>
+      </c>
+      <c r="CS5">
+        <f t="shared" si="91"/>
+        <v>-39.683945797708276</v>
+      </c>
+      <c r="CT5">
+        <f t="shared" si="91"/>
+        <v>-40.256806242521151</v>
+      </c>
+      <c r="CU5">
+        <f t="shared" si="91"/>
+        <v>-40.827675125496597</v>
+      </c>
+      <c r="CV5">
+        <f t="shared" si="91"/>
+        <v>-41.396575613237232</v>
+      </c>
+      <c r="CW5">
+        <f t="shared" si="91"/>
+        <v>-41.963530376114164</v>
+      </c>
+      <c r="CX5">
+        <f t="shared" si="91"/>
+        <v>-42.528561603941043</v>
+      </c>
+      <c r="CY5">
+        <f t="shared" si="91"/>
+        <v>-43.091691020995313</v>
+      </c>
+      <c r="CZ5">
+        <f t="shared" si="91"/>
+        <v>-43.652939900420208</v>
+      </c>
+      <c r="DA5">
+        <f t="shared" si="91"/>
+        <v>-44.212329078039176</v>
+      </c>
+    </row>
+    <row r="6" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="14">
+        <f>SQRT(C3*C3 + C4*C4)</f>
+        <v>401.1234224026316</v>
+      </c>
+      <c r="E6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F6">
+        <f>F4*SINH(($C$3-F5)/F4)</f>
+        <v>400.00999987501274</v>
+      </c>
+      <c r="G6">
+        <f t="shared" ref="G6:BR6" si="92">G4*SINH(($C$3-G5)/G4)</f>
+        <v>400.20994490392331</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="92"/>
+        <v>400.4097900901038</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="92"/>
+        <v>400.6095355829662</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="92"/>
+        <v>400.80918153156199</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="92"/>
+        <v>401.0087280845645</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="92"/>
+        <v>401.2081753902828</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="92"/>
+        <v>401.40752359665584</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="92"/>
+        <v>401.6067728512557</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="92"/>
+        <v>401.80592330128798</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="92"/>
+        <v>402.00497509359212</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="92"/>
+        <v>402.20392837464971</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="92"/>
+        <v>402.4027832905731</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="92"/>
+        <v>402.60153998711922</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="92"/>
+        <v>402.80019860968275</v>
+      </c>
+      <c r="U6">
+        <f t="shared" si="92"/>
+        <v>402.99875930330086</v>
+      </c>
+      <c r="V6">
+        <f t="shared" si="92"/>
+        <v>403.19722221265368</v>
+      </c>
+      <c r="W6">
+        <f t="shared" si="92"/>
+        <v>403.39558748206468</v>
+      </c>
+      <c r="X6">
+        <f t="shared" si="92"/>
+        <v>403.59385525550329</v>
+      </c>
+      <c r="Y6">
+        <f t="shared" si="92"/>
+        <v>403.79202567658541</v>
+      </c>
+      <c r="Z6">
+        <f t="shared" si="92"/>
+        <v>403.99009888857438</v>
+      </c>
+      <c r="AA6">
+        <f t="shared" si="92"/>
+        <v>404.18807503438296</v>
+      </c>
+      <c r="AB6">
+        <f t="shared" si="92"/>
+        <v>404.38595425657388</v>
+      </c>
+      <c r="AC6">
+        <f t="shared" si="92"/>
+        <v>404.58373669736153</v>
+      </c>
+      <c r="AD6">
+        <f t="shared" si="92"/>
+        <v>404.78142249861207</v>
+      </c>
+      <c r="AE6">
+        <f t="shared" si="92"/>
+        <v>404.9790118018463</v>
+      </c>
+      <c r="AF6">
+        <f t="shared" si="92"/>
+        <v>405.1765047482391</v>
+      </c>
+      <c r="AG6">
+        <f t="shared" si="92"/>
+        <v>405.37390147862271</v>
+      </c>
+      <c r="AH6">
+        <f t="shared" si="92"/>
+        <v>405.57120213348497</v>
+      </c>
+      <c r="AI6">
+        <f t="shared" si="92"/>
+        <v>405.76840685297316</v>
+      </c>
+      <c r="AJ6">
+        <f t="shared" si="92"/>
+        <v>405.96551577689445</v>
+      </c>
+      <c r="AK6">
+        <f t="shared" si="92"/>
+        <v>406.16252904471634</v>
+      </c>
+      <c r="AL6">
+        <f t="shared" si="92"/>
+        <v>406.35944679556786</v>
+      </c>
+      <c r="AM6">
+        <f t="shared" si="92"/>
+        <v>406.55626916824207</v>
+      </c>
+      <c r="AN6">
+        <f t="shared" si="92"/>
+        <v>406.7529963011952</v>
+      </c>
+      <c r="AO6">
+        <f t="shared" si="92"/>
+        <v>406.94962833254925</v>
+      </c>
+      <c r="AP6">
+        <f t="shared" si="92"/>
+        <v>407.14616540009314</v>
+      </c>
+      <c r="AQ6">
+        <f t="shared" si="92"/>
+        <v>407.34260764128265</v>
+      </c>
+      <c r="AR6">
+        <f t="shared" si="92"/>
+        <v>407.53895519324277</v>
+      </c>
+      <c r="AS6">
+        <f t="shared" si="92"/>
+        <v>407.73520819276803</v>
+      </c>
+      <c r="AT6">
+        <f t="shared" si="92"/>
+        <v>407.93136677632424</v>
+      </c>
+      <c r="AU6">
+        <f t="shared" si="92"/>
+        <v>408.12743108004884</v>
+      </c>
+      <c r="AV6">
+        <f t="shared" si="92"/>
+        <v>408.32340123975268</v>
+      </c>
+      <c r="AW6">
+        <f t="shared" si="92"/>
+        <v>408.51927739092071</v>
+      </c>
+      <c r="AX6">
+        <f t="shared" si="92"/>
+        <v>408.71505966871342</v>
+      </c>
+      <c r="AY6">
+        <f t="shared" si="92"/>
+        <v>408.91074820796786</v>
+      </c>
+      <c r="AZ6">
+        <f t="shared" si="92"/>
+        <v>409.10634314319788</v>
+      </c>
+      <c r="BA6">
+        <f t="shared" si="92"/>
+        <v>409.30184460859664</v>
+      </c>
+      <c r="BB6">
+        <f t="shared" si="92"/>
+        <v>409.49725273803728</v>
+      </c>
+      <c r="BC6">
+        <f t="shared" si="92"/>
+        <v>409.6925676650726</v>
+      </c>
+      <c r="BD6">
+        <f t="shared" si="92"/>
+        <v>409.88778952293757</v>
+      </c>
+      <c r="BE6">
+        <f t="shared" si="92"/>
+        <v>410.08291844455073</v>
+      </c>
+      <c r="BF6">
+        <f t="shared" si="92"/>
+        <v>410.27795456251386</v>
+      </c>
+      <c r="BG6">
+        <f t="shared" si="92"/>
+        <v>410.47289800911341</v>
+      </c>
+      <c r="BH6">
+        <f t="shared" si="92"/>
+        <v>410.66774891632281</v>
+      </c>
+      <c r="BI6">
+        <f t="shared" si="92"/>
+        <v>410.86250741580193</v>
+      </c>
+      <c r="BJ6">
+        <f t="shared" si="92"/>
+        <v>411.05717363889909</v>
+      </c>
+      <c r="BK6">
+        <f t="shared" si="92"/>
+        <v>411.25174771665098</v>
+      </c>
+      <c r="BL6">
+        <f t="shared" si="92"/>
+        <v>411.44622977978548</v>
+      </c>
+      <c r="BM6">
+        <f t="shared" si="92"/>
+        <v>411.64061995872061</v>
+      </c>
+      <c r="BN6">
+        <f t="shared" si="92"/>
+        <v>411.83491838356781</v>
+      </c>
+      <c r="BO6">
+        <f t="shared" si="92"/>
+        <v>412.02912518413052</v>
+      </c>
+      <c r="BP6">
+        <f t="shared" si="92"/>
+        <v>412.22324048990731</v>
+      </c>
+      <c r="BQ6">
+        <f t="shared" si="92"/>
+        <v>412.41726443009151</v>
+      </c>
+      <c r="BR6">
+        <f t="shared" si="92"/>
+        <v>412.61119713357294</v>
+      </c>
+      <c r="BS6">
+        <f t="shared" ref="BS6:DA6" si="93">BS4*SINH(($C$3-BS5)/BS4)</f>
+        <v>412.80503872893803</v>
+      </c>
+      <c r="BT6">
+        <f t="shared" si="93"/>
+        <v>412.99878934447241</v>
+      </c>
+      <c r="BU6">
+        <f t="shared" si="93"/>
+        <v>413.19244910816087</v>
+      </c>
+      <c r="BV6">
+        <f t="shared" si="93"/>
+        <v>413.3860181476872</v>
+      </c>
+      <c r="BW6">
+        <f t="shared" si="93"/>
+        <v>413.57949659043783</v>
+      </c>
+      <c r="BX6">
+        <f t="shared" si="93"/>
+        <v>413.77288456350055</v>
+      </c>
+      <c r="BY6">
+        <f t="shared" si="93"/>
+        <v>413.96618219366655</v>
+      </c>
+      <c r="BZ6">
+        <f t="shared" si="93"/>
+        <v>414.15938960743108</v>
+      </c>
+      <c r="CA6">
+        <f t="shared" si="93"/>
+        <v>414.35250693099482</v>
+      </c>
+      <c r="CB6">
+        <f t="shared" si="93"/>
+        <v>414.54553429026333</v>
+      </c>
+      <c r="CC6">
+        <f t="shared" si="93"/>
+        <v>414.73847181085091</v>
+      </c>
+      <c r="CD6">
+        <f t="shared" si="93"/>
+        <v>414.93131961807848</v>
+      </c>
+      <c r="CE6">
+        <f t="shared" si="93"/>
+        <v>415.12407783697631</v>
+      </c>
+      <c r="CF6">
+        <f t="shared" si="93"/>
+        <v>415.31674659228457</v>
+      </c>
+      <c r="CG6">
+        <f t="shared" si="93"/>
+        <v>415.50932600845425</v>
+      </c>
+      <c r="CH6">
+        <f t="shared" si="93"/>
+        <v>415.70181620964797</v>
+      </c>
+      <c r="CI6">
+        <f t="shared" si="93"/>
+        <v>415.89421731974096</v>
+      </c>
+      <c r="CJ6">
+        <f t="shared" si="93"/>
+        <v>416.08652946232235</v>
+      </c>
+      <c r="CK6">
+        <f t="shared" si="93"/>
+        <v>416.27875276069517</v>
+      </c>
+      <c r="CL6">
+        <f t="shared" si="93"/>
+        <v>416.47088733787876</v>
+      </c>
+      <c r="CM6">
+        <f t="shared" si="93"/>
+        <v>416.66293331660773</v>
+      </c>
+      <c r="CN6">
+        <f t="shared" si="93"/>
+        <v>416.85489081933525</v>
+      </c>
+      <c r="CO6">
+        <f t="shared" si="93"/>
+        <v>417.0467599682321</v>
+      </c>
+      <c r="CP6">
+        <f t="shared" si="93"/>
+        <v>417.23854088518704</v>
+      </c>
+      <c r="CQ6">
+        <f t="shared" si="93"/>
+        <v>417.430233691811</v>
+      </c>
+      <c r="CR6">
+        <f t="shared" si="93"/>
+        <v>417.62183850943438</v>
+      </c>
+      <c r="CS6">
+        <f t="shared" si="93"/>
+        <v>417.81335545910895</v>
+      </c>
+      <c r="CT6">
+        <f t="shared" si="93"/>
+        <v>418.00478466161121</v>
+      </c>
+      <c r="CU6">
+        <f t="shared" si="93"/>
+        <v>418.19612623743899</v>
+      </c>
+      <c r="CV6">
+        <f t="shared" si="93"/>
+        <v>418.38738030681566</v>
+      </c>
+      <c r="CW6">
+        <f t="shared" si="93"/>
+        <v>418.57854698968993</v>
+      </c>
+      <c r="CX6">
+        <f t="shared" si="93"/>
+        <v>418.76962640573623</v>
+      </c>
+      <c r="CY6">
+        <f t="shared" si="93"/>
+        <v>418.96061867435685</v>
+      </c>
+      <c r="CZ6">
+        <f t="shared" si="93"/>
+        <v>419.15152391468149</v>
+      </c>
+      <c r="DA6">
+        <f t="shared" si="93"/>
+        <v>419.34234224556928</v>
+      </c>
+    </row>
+    <row r="7" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7">
+        <f>F5+F6</f>
+        <v>429.89710180588088</v>
+      </c>
+      <c r="G7">
+        <f t="shared" ref="G7:AU7" si="94">G5+G6</f>
+        <v>428.47833020736311</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="94"/>
+        <v>427.30312412555332</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="94"/>
+        <v>426.22947248495592</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="94"/>
+        <v>425.22232423232481</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="94"/>
+        <v>424.26477463981274</v>
+      </c>
+      <c r="L7">
+        <f>L5+L6</f>
+        <v>423.34679386132228</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="94"/>
+        <v>422.461725382704</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="94"/>
+        <v>421.60482422312197</v>
+      </c>
+      <c r="O7">
+        <f t="shared" si="94"/>
+        <v>420.77253507089688</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="94"/>
+        <v>419.96209391651973</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="94"/>
+        <v>419.17128995367756</v>
+      </c>
+      <c r="R7">
+        <f t="shared" si="94"/>
+        <v>418.39831441595277</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="94"/>
+        <v>417.64165994827374</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="94"/>
+        <v>416.90005100516169</v>
+      </c>
+      <c r="U7">
+        <f t="shared" si="94"/>
+        <v>416.17239416406153</v>
+      </c>
+      <c r="V7">
+        <f t="shared" si="94"/>
+        <v>415.45774170148491</v>
+      </c>
+      <c r="W7">
+        <f t="shared" si="94"/>
+        <v>414.75526428082378</v>
+      </c>
+      <c r="X7">
+        <f t="shared" si="94"/>
+        <v>414.06423006881147</v>
+      </c>
+      <c r="Y7">
+        <f t="shared" si="94"/>
+        <v>413.38398849338608</v>
+      </c>
+      <c r="Z7">
+        <f t="shared" si="94"/>
+        <v>412.71395742082063</v>
+      </c>
+      <c r="AA7">
+        <f t="shared" si="94"/>
+        <v>412.05361289697925</v>
+      </c>
+      <c r="AB7">
+        <f t="shared" si="94"/>
+        <v>411.4024808420636</v>
+      </c>
+      <c r="AC7">
+        <f t="shared" si="94"/>
+        <v>410.76013025484474</v>
+      </c>
+      <c r="AD7">
+        <f t="shared" si="94"/>
+        <v>410.12616759824203</v>
+      </c>
+      <c r="AE7">
+        <f t="shared" si="94"/>
+        <v>409.50023212017345</v>
+      </c>
+      <c r="AF7">
+        <f t="shared" si="94"/>
+        <v>408.88199192265773</v>
+      </c>
+      <c r="AG7">
+        <f t="shared" si="94"/>
+        <v>408.27114063531985</v>
+      </c>
+      <c r="AH7">
+        <f t="shared" si="94"/>
+        <v>407.66739458140364</v>
+      </c>
+      <c r="AI7">
+        <f t="shared" si="94"/>
+        <v>407.07049034838633</v>
+      </c>
+      <c r="AJ7">
+        <f t="shared" si="94"/>
+        <v>406.48018269345766</v>
+      </c>
+      <c r="AK7">
+        <f t="shared" si="94"/>
+        <v>405.89624272808101</v>
+      </c>
+      <c r="AL7">
+        <f t="shared" si="94"/>
+        <v>405.31845633664477</v>
+      </c>
+      <c r="AM7">
+        <f t="shared" si="94"/>
+        <v>404.74662279264732</v>
+      </c>
+      <c r="AN7">
+        <f t="shared" si="94"/>
+        <v>404.18055354249708</v>
+      </c>
+      <c r="AO7">
+        <f t="shared" si="94"/>
+        <v>403.6200711322972</v>
+      </c>
+      <c r="AP7">
+        <f t="shared" si="94"/>
+        <v>403.06500825719638</v>
+      </c>
+      <c r="AQ7">
+        <f t="shared" si="94"/>
+        <v>402.5152069162915</v>
+      </c>
+      <c r="AR7">
+        <f t="shared" si="94"/>
+        <v>401.97051765882992</v>
+      </c>
+      <c r="AS7">
+        <f t="shared" si="94"/>
+        <v>401.43079890970165</v>
+      </c>
+      <c r="AT7">
+        <f t="shared" si="94"/>
+        <v>400.89591636406436</v>
+      </c>
+      <c r="AU7">
+        <f t="shared" si="94"/>
+        <v>400.36574244246265</v>
+      </c>
+      <c r="AV7">
+        <f t="shared" ref="AV7:BH7" si="95">AV5+AV6</f>
+        <v>399.84015579907049</v>
+      </c>
+      <c r="AW7">
+        <f t="shared" si="95"/>
+        <v>399.31904087673507</v>
+      </c>
+      <c r="AX7">
+        <f t="shared" si="95"/>
+        <v>398.80228750338358</v>
+      </c>
+      <c r="AY7">
+        <f t="shared" si="95"/>
+        <v>398.28979052509555</v>
+      </c>
+      <c r="AZ7">
+        <f t="shared" si="95"/>
+        <v>397.78144947176798</v>
+      </c>
+      <c r="BA7">
+        <f t="shared" si="95"/>
+        <v>397.27716825183592</v>
+      </c>
+      <c r="BB7">
+        <f t="shared" si="95"/>
+        <v>396.77685487295531</v>
+      </c>
+      <c r="BC7">
+        <f t="shared" si="95"/>
+        <v>396.28042118594601</v>
+      </c>
+      <c r="BD7">
+        <f t="shared" si="95"/>
+        <v>395.78778264962671</v>
+      </c>
+      <c r="BE7">
+        <f t="shared" si="95"/>
+        <v>395.29885811444956</v>
+      </c>
+      <c r="BF7">
+        <f t="shared" si="95"/>
+        <v>394.8135696230928</v>
+      </c>
+      <c r="BG7">
+        <f t="shared" si="95"/>
+        <v>394.33184222638386</v>
+      </c>
+      <c r="BH7">
+        <f t="shared" si="95"/>
+        <v>393.85360381310738</v>
+      </c>
+      <c r="BI7">
+        <f t="shared" ref="BI7:BZ7" si="96">BI5+BI6</f>
+        <v>393.37878495241006</v>
+      </c>
+      <c r="BJ7">
+        <f t="shared" si="96"/>
+        <v>392.90731874766158</v>
+      </c>
+      <c r="BK7">
+        <f t="shared" si="96"/>
+        <v>392.43914070074658</v>
+      </c>
+      <c r="BL7">
+        <f t="shared" si="96"/>
+        <v>391.97418858587639</v>
+      </c>
+      <c r="BM7">
+        <f t="shared" si="96"/>
+        <v>391.51240233209541</v>
+      </c>
+      <c r="BN7">
+        <f t="shared" si="96"/>
+        <v>391.05372391375181</v>
+      </c>
+      <c r="BO7">
+        <f t="shared" si="96"/>
+        <v>390.59809724826209</v>
+      </c>
+      <c r="BP7">
+        <f t="shared" si="96"/>
+        <v>390.14546810058005</v>
+      </c>
+      <c r="BQ7">
+        <f t="shared" si="96"/>
+        <v>389.69578399382192</v>
+      </c>
+      <c r="BR7">
+        <f t="shared" si="96"/>
+        <v>389.24899412556567</v>
+      </c>
+      <c r="BS7">
+        <f t="shared" si="96"/>
+        <v>388.80504928937631</v>
+      </c>
+      <c r="BT7">
+        <f t="shared" si="96"/>
+        <v>388.36390180116098</v>
+      </c>
+      <c r="BU7">
+        <f t="shared" si="96"/>
+        <v>387.92550542998197</v>
+      </c>
+      <c r="BV7">
+        <f t="shared" si="96"/>
+        <v>387.48981533299832</v>
+      </c>
+      <c r="BW7">
+        <f t="shared" si="96"/>
+        <v>387.05678799423578</v>
+      </c>
+      <c r="BX7">
+        <f t="shared" si="96"/>
+        <v>386.62638116690022</v>
+      </c>
+      <c r="BY7">
+        <f t="shared" si="96"/>
+        <v>386.19855381898839</v>
+      </c>
+      <c r="BZ7">
+        <f t="shared" si="96"/>
+        <v>385.77326608196051</v>
+      </c>
+      <c r="CA7">
+        <f t="shared" ref="CA7:DA7" si="97">CA5+CA6</f>
+        <v>385.3504792022635</v>
+      </c>
+      <c r="CB7">
+        <f t="shared" si="97"/>
+        <v>384.93015549550728</v>
+      </c>
+      <c r="CC7">
+        <f t="shared" si="97"/>
+        <v>384.51225830312097</v>
+      </c>
+      <c r="CD7">
+        <f t="shared" si="97"/>
+        <v>384.09675195131456</v>
+      </c>
+      <c r="CE7">
+        <f t="shared" si="97"/>
+        <v>383.68360171220331</v>
+      </c>
+      <c r="CF7">
+        <f t="shared" si="97"/>
+        <v>383.27277376694923</v>
+      </c>
+      <c r="CG7">
+        <f t="shared" si="97"/>
+        <v>382.86423517079197</v>
+      </c>
+      <c r="CH7">
+        <f t="shared" si="97"/>
+        <v>382.45795381984976</v>
+      </c>
+      <c r="CI7">
+        <f t="shared" si="97"/>
+        <v>382.0538984195793</v>
+      </c>
+      <c r="CJ7">
+        <f t="shared" si="97"/>
+        <v>381.65203845479306</v>
+      </c>
+      <c r="CK7">
+        <f t="shared" si="97"/>
+        <v>381.25234416113744</v>
+      </c>
+      <c r="CL7">
+        <f t="shared" si="97"/>
+        <v>380.85478649794709</v>
+      </c>
+      <c r="CM7">
+        <f t="shared" si="97"/>
+        <v>380.45933712238769</v>
+      </c>
+      <c r="CN7">
+        <f t="shared" si="97"/>
+        <v>380.06596836482009</v>
+      </c>
+      <c r="CO7">
+        <f t="shared" si="97"/>
+        <v>379.67465320530493</v>
+      </c>
+      <c r="CP7">
+        <f t="shared" si="97"/>
+        <v>379.28536525118886</v>
+      </c>
+      <c r="CQ7">
+        <f t="shared" si="97"/>
+        <v>378.89807871571247</v>
+      </c>
+      <c r="CR7">
+        <f t="shared" si="97"/>
+        <v>378.51276839757332</v>
+      </c>
+      <c r="CS7">
+        <f t="shared" si="97"/>
+        <v>378.1294096614007</v>
+      </c>
+      <c r="CT7">
+        <f t="shared" si="97"/>
+        <v>377.74797841909003</v>
+      </c>
+      <c r="CU7">
+        <f t="shared" si="97"/>
+        <v>377.36845111194236</v>
+      </c>
+      <c r="CV7">
+        <f t="shared" si="97"/>
+        <v>376.99080469357841</v>
+      </c>
+      <c r="CW7">
+        <f t="shared" si="97"/>
+        <v>376.61501661357579</v>
+      </c>
+      <c r="CX7">
+        <f t="shared" si="97"/>
+        <v>376.24106480179518</v>
+      </c>
+      <c r="CY7">
+        <f t="shared" si="97"/>
+        <v>375.86892765336154</v>
+      </c>
+      <c r="CZ7">
+        <f t="shared" si="97"/>
+        <v>375.49858401426127</v>
+      </c>
+      <c r="DA7">
+        <f t="shared" si="97"/>
+        <v>375.13001316753014</v>
+      </c>
+    </row>
+    <row r="8" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8">
+        <f>ABS(F7-$C$5)</f>
+        <v>9.8971018058808795</v>
+      </c>
+      <c r="G8">
+        <f t="shared" ref="G8:AU8" si="98">ABS(G7-$C$5)</f>
+        <v>8.4783302073631148</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="98"/>
+        <v>7.3031241255533246</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="98"/>
+        <v>6.2294724849559202</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="98"/>
+        <v>5.2223242323248087</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="98"/>
+        <v>4.2647746398127424</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="98"/>
+        <v>3.3467938613222827</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="98"/>
+        <v>2.4617253827040031</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="98"/>
+        <v>1.604824223121966</v>
+      </c>
+      <c r="O8">
+        <f t="shared" si="98"/>
+        <v>0.77253507089687901</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="98"/>
+        <v>3.7906083480265806E-2</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="98"/>
+        <v>0.82871004632244194</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="98"/>
+        <v>1.6016855840472317</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="98"/>
+        <v>2.3583400517262589</v>
+      </c>
+      <c r="T8">
+        <f t="shared" si="98"/>
+        <v>3.0999489948383143</v>
+      </c>
+      <c r="U8">
+        <f t="shared" si="98"/>
+        <v>3.8276058359384706</v>
+      </c>
+      <c r="V8">
+        <f t="shared" si="98"/>
+        <v>4.5422582985150939</v>
+      </c>
+      <c r="W8">
+        <f t="shared" si="98"/>
+        <v>5.2447357191762194</v>
+      </c>
+      <c r="X8">
+        <f t="shared" si="98"/>
+        <v>5.9357699311885312</v>
+      </c>
+      <c r="Y8">
+        <f t="shared" si="98"/>
+        <v>6.6160115066139156</v>
+      </c>
+      <c r="Z8">
+        <f t="shared" si="98"/>
+        <v>7.2860425791793659</v>
+      </c>
+      <c r="AA8">
+        <f t="shared" si="98"/>
+        <v>7.9463871030207542</v>
+      </c>
+      <c r="AB8">
+        <f t="shared" si="98"/>
+        <v>8.5975191579364036</v>
+      </c>
+      <c r="AC8">
+        <f t="shared" si="98"/>
+        <v>9.2398697451552607</v>
+      </c>
+      <c r="AD8">
+        <f t="shared" si="98"/>
+        <v>9.8738324017579657</v>
+      </c>
+      <c r="AE8">
+        <f t="shared" si="98"/>
+        <v>10.49976787982655</v>
+      </c>
+      <c r="AF8">
+        <f t="shared" si="98"/>
+        <v>11.118008077342267</v>
+      </c>
+      <c r="AG8">
+        <f t="shared" si="98"/>
+        <v>11.728859364680147</v>
+      </c>
+      <c r="AH8">
+        <f t="shared" si="98"/>
+        <v>12.332605418596359</v>
+      </c>
+      <c r="AI8">
+        <f t="shared" si="98"/>
+        <v>12.929509651613671</v>
+      </c>
+      <c r="AJ8">
+        <f t="shared" si="98"/>
+        <v>13.519817306542336</v>
+      </c>
+      <c r="AK8">
+        <f t="shared" si="98"/>
+        <v>14.103757271918994</v>
+      </c>
+      <c r="AL8">
+        <f t="shared" si="98"/>
+        <v>14.681543663355228</v>
+      </c>
+      <c r="AM8">
+        <f t="shared" si="98"/>
+        <v>15.253377207352685</v>
+      </c>
+      <c r="AN8">
+        <f t="shared" si="98"/>
+        <v>15.81944645750292</v>
+      </c>
+      <c r="AO8">
+        <f t="shared" si="98"/>
+        <v>16.379928867702802</v>
+      </c>
+      <c r="AP8">
+        <f t="shared" si="98"/>
+        <v>16.934991742803618</v>
+      </c>
+      <c r="AQ8">
+        <f t="shared" si="98"/>
+        <v>17.484793083708496</v>
+      </c>
+      <c r="AR8">
+        <f t="shared" si="98"/>
+        <v>18.02948234117008</v>
+      </c>
+      <c r="AS8">
+        <f t="shared" si="98"/>
+        <v>18.56920109029835</v>
+      </c>
+      <c r="AT8">
+        <f t="shared" si="98"/>
+        <v>19.104083635935638</v>
+      </c>
+      <c r="AU8">
+        <f t="shared" si="98"/>
+        <v>19.634257557537353</v>
+      </c>
+      <c r="AV8">
+        <f t="shared" ref="AV8" si="99">ABS(AV7-$C$5)</f>
+        <v>20.159844200929513</v>
+      </c>
+      <c r="AW8">
+        <f t="shared" ref="AW8" si="100">ABS(AW7-$C$5)</f>
+        <v>20.680959123264927</v>
+      </c>
+      <c r="AX8">
+        <f t="shared" ref="AX8" si="101">ABS(AX7-$C$5)</f>
+        <v>21.197712496616418</v>
+      </c>
+      <c r="AY8">
+        <f t="shared" ref="AY8" si="102">ABS(AY7-$C$5)</f>
+        <v>21.710209474904445</v>
+      </c>
+      <c r="AZ8">
+        <f t="shared" ref="AZ8" si="103">ABS(AZ7-$C$5)</f>
+        <v>22.218550528232015</v>
+      </c>
+      <c r="BA8">
+        <f t="shared" ref="BA8" si="104">ABS(BA7-$C$5)</f>
+        <v>22.722831748164083</v>
+      </c>
+      <c r="BB8">
+        <f t="shared" ref="BB8" si="105">ABS(BB7-$C$5)</f>
+        <v>23.223145127044688</v>
+      </c>
+      <c r="BC8">
+        <f t="shared" ref="BC8" si="106">ABS(BC7-$C$5)</f>
+        <v>23.719578814053989</v>
+      </c>
+      <c r="BD8">
+        <f t="shared" ref="BD8" si="107">ABS(BD7-$C$5)</f>
+        <v>24.212217350373294</v>
+      </c>
+      <c r="BE8">
+        <f t="shared" ref="BE8" si="108">ABS(BE7-$C$5)</f>
+        <v>24.701141885550442</v>
+      </c>
+      <c r="BF8">
+        <f t="shared" ref="BF8" si="109">ABS(BF7-$C$5)</f>
+        <v>25.186430376907197</v>
+      </c>
+      <c r="BG8">
+        <f t="shared" ref="BG8" si="110">ABS(BG7-$C$5)</f>
+        <v>25.668157773616144</v>
+      </c>
+      <c r="BH8">
+        <f t="shared" ref="BH8" si="111">ABS(BH7-$C$5)</f>
+        <v>26.146396186892616</v>
+      </c>
+      <c r="BI8">
+        <f t="shared" ref="BI8" si="112">ABS(BI7-$C$5)</f>
+        <v>26.621215047589942</v>
+      </c>
+      <c r="BJ8">
+        <f t="shared" ref="BJ8" si="113">ABS(BJ7-$C$5)</f>
+        <v>27.092681252338423</v>
+      </c>
+      <c r="BK8">
+        <f t="shared" ref="BK8" si="114">ABS(BK7-$C$5)</f>
+        <v>27.560859299253423</v>
+      </c>
+      <c r="BL8">
+        <f t="shared" ref="BL8" si="115">ABS(BL7-$C$5)</f>
+        <v>28.025811414123609</v>
+      </c>
+      <c r="BM8">
+        <f t="shared" ref="BM8" si="116">ABS(BM7-$C$5)</f>
+        <v>28.487597667904595</v>
+      </c>
+      <c r="BN8">
+        <f t="shared" ref="BN8" si="117">ABS(BN7-$C$5)</f>
+        <v>28.94627608624819</v>
+      </c>
+      <c r="BO8">
+        <f t="shared" ref="BO8" si="118">ABS(BO7-$C$5)</f>
+        <v>29.401902751737907</v>
+      </c>
+      <c r="BP8">
+        <f t="shared" ref="BP8" si="119">ABS(BP7-$C$5)</f>
+        <v>29.854531899419953</v>
+      </c>
+      <c r="BQ8">
+        <f t="shared" ref="BQ8" si="120">ABS(BQ7-$C$5)</f>
+        <v>30.304216006178081</v>
+      </c>
+      <c r="BR8">
+        <f t="shared" ref="BR8" si="121">ABS(BR7-$C$5)</f>
+        <v>30.751005874434327</v>
+      </c>
+      <c r="BS8">
+        <f t="shared" ref="BS8" si="122">ABS(BS7-$C$5)</f>
+        <v>31.194950710623687</v>
+      </c>
+      <c r="BT8">
+        <f t="shared" ref="BT8" si="123">ABS(BT7-$C$5)</f>
+        <v>31.636098198839022</v>
+      </c>
+      <c r="BU8">
+        <f t="shared" ref="BU8" si="124">ABS(BU7-$C$5)</f>
+        <v>32.074494570018032</v>
+      </c>
+      <c r="BV8">
+        <f t="shared" ref="BV8" si="125">ABS(BV7-$C$5)</f>
+        <v>32.510184667001681</v>
+      </c>
+      <c r="BW8">
+        <f t="shared" ref="BW8" si="126">ABS(BW7-$C$5)</f>
+        <v>32.943212005764224</v>
+      </c>
+      <c r="BX8">
+        <f t="shared" ref="BX8" si="127">ABS(BX7-$C$5)</f>
+        <v>33.373618833099783</v>
+      </c>
+      <c r="BY8">
+        <f t="shared" ref="BY8" si="128">ABS(BY7-$C$5)</f>
+        <v>33.801446181011613</v>
+      </c>
+      <c r="BZ8">
+        <f t="shared" ref="BZ8" si="129">ABS(BZ7-$C$5)</f>
+        <v>34.226733918039486</v>
+      </c>
+      <c r="CA8">
+        <f t="shared" ref="CA8" si="130">ABS(CA7-$C$5)</f>
+        <v>34.6495207977365</v>
+      </c>
+      <c r="CB8">
+        <f t="shared" ref="CB8" si="131">ABS(CB7-$C$5)</f>
+        <v>35.069844504492721</v>
+      </c>
+      <c r="CC8">
+        <f t="shared" ref="CC8" si="132">ABS(CC7-$C$5)</f>
+        <v>35.487741696879027</v>
+      </c>
+      <c r="CD8">
+        <f t="shared" ref="CD8" si="133">ABS(CD7-$C$5)</f>
+        <v>35.903248048685441</v>
+      </c>
+      <c r="CE8">
+        <f t="shared" ref="CE8" si="134">ABS(CE7-$C$5)</f>
+        <v>36.316398287796687</v>
+      </c>
+      <c r="CF8">
+        <f t="shared" ref="CF8" si="135">ABS(CF7-$C$5)</f>
+        <v>36.727226233050771</v>
+      </c>
+      <c r="CG8">
+        <f t="shared" ref="CG8" si="136">ABS(CG7-$C$5)</f>
+        <v>37.135764829208028</v>
+      </c>
+      <c r="CH8">
+        <f t="shared" ref="CH8" si="137">ABS(CH7-$C$5)</f>
+        <v>37.542046180150237</v>
+      </c>
+      <c r="CI8">
+        <f t="shared" ref="CI8" si="138">ABS(CI7-$C$5)</f>
+        <v>37.946101580420702</v>
+      </c>
+      <c r="CJ8">
+        <f t="shared" ref="CJ8" si="139">ABS(CJ7-$C$5)</f>
+        <v>38.347961545206942</v>
+      </c>
+      <c r="CK8">
+        <f t="shared" ref="CK8" si="140">ABS(CK7-$C$5)</f>
+        <v>38.747655838862556</v>
+      </c>
+      <c r="CL8">
+        <f t="shared" ref="CL8" si="141">ABS(CL7-$C$5)</f>
+        <v>39.145213502052911</v>
+      </c>
+      <c r="CM8">
+        <f t="shared" ref="CM8" si="142">ABS(CM7-$C$5)</f>
+        <v>39.540662877612306</v>
+      </c>
+      <c r="CN8">
+        <f t="shared" ref="CN8" si="143">ABS(CN7-$C$5)</f>
+        <v>39.934031635179906</v>
+      </c>
+      <c r="CO8">
+        <f t="shared" ref="CO8" si="144">ABS(CO7-$C$5)</f>
+        <v>40.325346794695065</v>
+      </c>
+      <c r="CP8">
+        <f t="shared" ref="CP8" si="145">ABS(CP7-$C$5)</f>
+        <v>40.714634748811136</v>
+      </c>
+      <c r="CQ8">
+        <f t="shared" ref="CQ8" si="146">ABS(CQ7-$C$5)</f>
+        <v>41.101921284287528</v>
+      </c>
+      <c r="CR8">
+        <f t="shared" ref="CR8" si="147">ABS(CR7-$C$5)</f>
+        <v>41.487231602426675</v>
+      </c>
+      <c r="CS8">
+        <f t="shared" ref="CS8" si="148">ABS(CS7-$C$5)</f>
+        <v>41.8705903385993</v>
+      </c>
+      <c r="CT8">
+        <f t="shared" ref="CT8" si="149">ABS(CT7-$C$5)</f>
+        <v>42.252021580909968</v>
+      </c>
+      <c r="CU8">
+        <f t="shared" ref="CU8" si="150">ABS(CU7-$C$5)</f>
+        <v>42.631548888057637</v>
+      </c>
+      <c r="CV8">
+        <f t="shared" ref="CV8" si="151">ABS(CV7-$C$5)</f>
+        <v>43.009195306421589</v>
+      </c>
+      <c r="CW8">
+        <f t="shared" ref="CW8" si="152">ABS(CW7-$C$5)</f>
+        <v>43.38498338642421</v>
+      </c>
+      <c r="CX8">
+        <f t="shared" ref="CX8" si="153">ABS(CX7-$C$5)</f>
+        <v>43.758935198204824</v>
+      </c>
+      <c r="CY8">
+        <f t="shared" ref="CY8" si="154">ABS(CY7-$C$5)</f>
+        <v>44.131072346638462</v>
+      </c>
+      <c r="CZ8">
+        <f t="shared" ref="CZ8" si="155">ABS(CZ7-$C$5)</f>
+        <v>44.501415985738731</v>
+      </c>
+      <c r="DA8">
+        <f t="shared" ref="DA8" si="156">ABS(DA7-$C$5)</f>
+        <v>44.869986832469863</v>
+      </c>
+    </row>
+    <row r="9" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9">
+        <f>MIN(F8:AU8)</f>
+        <v>3.7906083480265806E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10">
+        <f>_xlfn.XMATCH(C9,F8:AU8)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" cm="1">
+        <f t="array" ref="C11">INDEX(F4:AU4,C$10)</f>
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="E11" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA11">
+        <f>AA4*ACOSH((($C$4+AA4)/AA4))</f>
+        <v>22.134462137403741</v>
+      </c>
+    </row>
+    <row r="12" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" cm="1">
+        <f t="array" ref="C12">INDEX(F5:AU5,C$10)</f>
+        <v>17.957118822927626</v>
+      </c>
+    </row>
+    <row r="13" spans="2:105" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" cm="1">
+        <f t="array" ref="C13">INDEX(F6:AU6,C10)</f>
+        <v>402.00497509359212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>